<commit_message>
Add pins - 2026-07-14 07:52 UTC
</commit_message>
<xml_diff>
--- a/pins/pin_links.xlsx
+++ b/pins/pin_links.xlsx
@@ -467,12 +467,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cancer Survivor Uses Her Diagnosis To Justify A Hall Pass Request That Ends Her 20-Year Marriage</t>
+          <t>55 Doctors Reveal The Health Problems Showing Up More Than Ever Before</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0001-cancer-survivor-uses-her-diagnosis-to-justify-a-hall-pass-re.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0001-55-doctors-reveal-the-health-problems-showing-up-more-than-e.jpg</t>
         </is>
       </c>
     </row>
@@ -482,12 +482,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>15 Real-Life Bizarre Accidents That Sound Fake, But Ultimately Took The Lives Of Innocent People</t>
+          <t>“This Hurts My Eyes”: 50 Attempts That Were Made But They Were Not Good Enough (New Pics)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0002-15-real-life-bizarre-accidents-that-sound-fake-but-ultimatel.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0002-this-hurts-my-eyes-50-attempts-that-were-made-but-they-were-.jpg</t>
         </is>
       </c>
     </row>
@@ -497,12 +497,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>“Apologize For What?” GF Accuses BF Of Cheating After He Bearhugged Friend Having Breakdown</t>
+          <t>Bride Asks Mom Why She Wants The Wedding Delayed, Doesn’t Like The Answer</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0003-apologize-for-what-gf-accuses-bf-of-cheating-after-he-bearhu.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0003-bride-asks-mom-why-she-wants-the-wedding-delayed-doesnt-like.jpg</t>
         </is>
       </c>
     </row>
@@ -512,12 +512,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Family’s Goodbye Visit Turns Chaotic When Grandma Won’t Leave And Takes Hold Of Toddler</t>
+          <t>Woman Refuses To Spend Vacation Babysitting Sister’s Kids, Family Drama Follows</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0004-familys-goodbye-visit-turns-chaotic-when-grandma-wont-leave-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0004-woman-refuses-to-spend-vacation-babysitting-sisters-kids-fam.jpg</t>
         </is>
       </c>
     </row>
@@ -527,12 +527,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>21 Prime Day Outdoor And Backyard Essentials That Are About To Make Your Summer So Much Better</t>
+          <t>If You Answer All 21 General Knowledge Questions, You’re Basically A Walking Encyclopedia</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0005-21-prime-day-outdoor-and-backyard-essentials-that-are-about-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0005-if-you-answer-all-21-general-knowledge-questions-youre-basic.jpg</t>
         </is>
       </c>
     </row>
@@ -542,12 +542,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>“This Isn’t Over”: In-Laws Treat Couple’s Home As Redecoration Project, Mad When DIL Bans Them</t>
+          <t>Daily Guess The Timeline Game #087 (Jun 18, 2026)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0006-this-isnt-over-in-laws-treat-couples-home-as-redecoration-pr.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0006-daily-guess-the-timeline-game-087-jun-18-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -557,12 +557,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>After Weeks Of Planning And Childcare Arrangements, Woman Discovers Group Hike Wasn’t Really A Hike</t>
+          <t>Narcissistic Parents: A Survival Guide for Adult Children</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0007-after-weeks-of-planning-and-childcare-arrangements-woman-dis.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0007-narcissistic-parents-a-survival-guide-for-adult-children.jpg</t>
         </is>
       </c>
     </row>
@@ -572,12 +572,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>“[AITJ] For Turning Down A Family Vacation Because I Would Have To Pay And My Sister Wouldn’t?”</t>
+          <t>Only A Well-Read Person Can Answer All 20 Of These Questions On Classic Literature</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0008-aitj-for-turning-down-a-family-vacation-because-i-would-have.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0008-only-a-well-read-person-can-answer-all-20-of-these-questions.jpg</t>
         </is>
       </c>
     </row>
@@ -587,12 +587,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>“Am I The Jerk For Calling The Cops To Remove My Ex-Wife From My Home?”</t>
+          <t>Shelter Dogs Are Finding New Homes After This Man Gives Them Backpack Rides Around NYC</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0009-am-i-the-jerk-for-calling-the-cops-to-remove-my-ex-wife-from.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0009-shelter-dogs-are-finding-new-homes-after-this-man-gives-them.jpg</t>
         </is>
       </c>
     </row>
@@ -602,12 +602,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>“Can’t Expect Much”: Guy Is Shocked Kids Don’t See Him As A Father, Ex-Wife Tells Him Exactly Why</t>
+          <t>Daily Guess The Country Game #033 (Jun 18, 2026)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0010-cant-expect-much-guy-is-shocked-kids-dont-see-him-as-a-fathe.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0010-daily-guess-the-country-game-033-jun-18-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -617,12 +617,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Man Feels Abandoned After Fainting At Music Festival, Starts Wondering If He Should Call Off Wedding</t>
+          <t>31 Clever And Absurd Comics By John Atkinson That Put A Weird Spin On Random Everyday Thoughts</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0011-man-feels-abandoned-after-fainting-at-music-festival-starts-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0011-31-clever-and-absurd-comics-by-john-atkinson-that-put-a-weir.jpg</t>
         </is>
       </c>
     </row>
@@ -632,12 +632,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>58 Times Kids Were So Betrayed By Their Parents, They Never Saw Them Again</t>
+          <t>This Cartoonist Created 39 Weird, Dark Humor Comics Full Of Bizarre Twists</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0012-58-times-kids-were-so-betrayed-by-their-parents-they-never-s.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0012-this-cartoonist-created-39-weird-dark-humor-comics-full-of-b.jpg</t>
         </is>
       </c>
     </row>
@@ -647,12 +647,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Childfree Woman’s Response To One Pregnancy Comment Left An Entire Wedding Table Stunned</t>
+          <t>32 Wild And Unsettling Vintage Toy Designs By Shampoooty That Defy Norms</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0013-childfree-womans-response-to-one-pregnancy-comment-left-an-e.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0013-32-wild-and-unsettling-vintage-toy-designs-by-shampoooty-tha.jpg</t>
         </is>
       </c>
     </row>
@@ -662,12 +662,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>69 People Who Quit Their Jobs To Travel Share If They Regret It Now</t>
+          <t>The Best 100 Comics By Stephen Beals About Retail, Work Stress, And Customer Interactions (Part 1)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0014-69-people-who-quit-their-jobs-to-travel-share-if-they-regret.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0014-the-best-100-comics-by-stephen-beals-about-retail-work-stres.jpg</t>
         </is>
       </c>
     </row>
@@ -677,12 +677,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>“Which Ancient Civilization Would You Have Thrived In?”: Find Out In 27 Questions</t>
+          <t>Daily Word Search Game #031 (Jun 18, 2026)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0015-which-ancient-civilization-would-you-have-thrived-in-find-ou.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0015-daily-word-search-game-031-jun-18-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -692,12 +692,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>53 Pieces Of History That Sent People Down A Rabbit Hole</t>
+          <t>33 Wholesome Posts About Men Defining Masculinity In Their Own Way</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0016-53-pieces-of-history-that-sent-people-down-a-rabbit-hole.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0016-33-wholesome-posts-about-men-defining-masculinity-in-their-o.jpg</t>
         </is>
       </c>
     </row>
@@ -707,12 +707,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>87 Myths About Men And Women That People Refuse To Let Go Of</t>
+          <t>27 Times A Perfectly Normal Person Turned Out To Have A Dark Side</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0017-87-myths-about-men-and-women-that-people-refuse-to-let-go-of.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0017-27-times-a-perfectly-normal-person-turned-out-to-have-a-dark.jpg</t>
         </is>
       </c>
     </row>
@@ -722,12 +722,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>33 Unbelievably Creepy Things That Happened To People</t>
+          <t>69 “Comments You Can Hear” That Practically Read Themselves Out Loud</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0018-33-unbelievably-creepy-things-that-happened-to-people.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0018-69-comments-you-can-hear-that-practically-read-themselves-ou.jpg</t>
         </is>
       </c>
     </row>
@@ -737,12 +737,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Daily Guess The Timeline Game #093 (Jun 24, 2026)</t>
+          <t>Doctor Exposes Shocking Studies On Women’s Health, And People Are Absolutely Furious</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0019-daily-guess-the-timeline-game-093-jun-24-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0019-doctor-exposes-shocking-studies-on-womens-health-and-people-.jpg</t>
         </is>
       </c>
     </row>
@@ -752,12 +752,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bombshell Report Reveals Jennifer Aniston And Other A-Listers Involved In Hollywood Voting Scandal</t>
+          <t>This Artist Captures The Chaos, Charm, And Confidence Of Pomeranians In 40 Comics</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0020-bombshell-report-reveals-jennifer-aniston-and-other-a-lister.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0020-this-artist-captures-the-chaos-charm-and-confidence-of-pomer.jpg</t>
         </is>
       </c>
     </row>
@@ -767,12 +767,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>91 Historic Photos That Show How Much These Places Have Changed</t>
+          <t>Daily Guess The Famous Person Game #092 (Jun 18, 2026)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0021-91-historic-photos-that-show-how-much-these-places-have-chan.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0021-daily-guess-the-famous-person-game-092-jun-18-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -782,12 +782,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Woman Gets Engaged, Twin Sister’s First Question Isn’t About The Wedding</t>
+          <t>49 Last Minute Father’s Day Gifts That Are So Good Dad Will Never Know You Ordered Them Yesterday</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0022-woman-gets-engaged-twin-sisters-first-question-isnt-about-th.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0022-49-last-minute-fathers-day-gifts-that-are-so-good-dad-will-n.jpg</t>
         </is>
       </c>
     </row>
@@ -797,12 +797,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>57 Internet Posts That Aged Better Than Anyone Could Have Imagined (New Pics)</t>
+          <t>40 Unsettling True Stories From “Oddly Horrifying” That Show How Dark The Real World Can Be (New Pics)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0023-57-internet-posts-that-aged-better-than-anyone-could-have-im.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0023-40-unsettling-true-stories-from-oddly-horrifying-that-show-h.jpg</t>
         </is>
       </c>
     </row>
@@ -812,12 +812,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>After Years Of Silence, Joe Manganiello Reveals His Life-Threatening Health Battle And Major ‘Amputation’</t>
+          <t>30 Wild Stories Of People Whose Double Lives Eventually Caught Up With Them</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0024-after-years-of-silence-joe-manganiello-reveals-his-life-thre.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0024-30-wild-stories-of-people-whose-double-lives-eventually-caug.jpg</t>
         </is>
       </c>
     </row>
@@ -827,12 +827,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Daily Guess The Country Game #039 (Jun 24, 2026)</t>
+          <t>“May God Punish You For How You Treated Me”: 76 Online Reviews That Are Funnier Than They Should Be</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0025-daily-guess-the-country-game-039-jun-24-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0025-may-god-punish-you-for-how-you-treated-me-76-online-reviews-.jpg</t>
         </is>
       </c>
     </row>
@@ -842,12 +842,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>57 Incredible Photos Shared By The ‘Raw Oceanlife’ Page That Capture The Wild Beauty Of The Deep Blue Sea</t>
+          <t>“What Is The Dumbest Thing You Have Been Told Is Not Manly Or Not Feminine?” (62 Answers)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0026-57-incredible-photos-shared-by-the-raw-oceanlife-page-that-c.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0026-what-is-the-dumbest-thing-you-have-been-told-is-not-manly-or.jpg</t>
         </is>
       </c>
     </row>
@@ -857,12 +857,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Artist Creates 39 Hilarious Comics About Friendship, Dating, And Everyday Life</t>
+          <t>Guy Dangles Engagement Ring To Get GF To Share Authorship Of Her Book, Won’t Take No For An Answer</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0027-artist-creates-39-hilarious-comics-about-friendship-dating-a.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0027-guy-dangles-engagement-ring-to-get-gf-to-share-authorship-of.jpg</t>
         </is>
       </c>
     </row>
@@ -872,12 +872,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>30 New “Off The Leash” Comics That Perfectly Capture Life With Dogs</t>
+          <t>Man Walks In On Gym Bros Hooking Up In The Steam Room, Gets Blamed For Ruining Their Alpha Image</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0028-30-new-off-the-leash-comics-that-perfectly-capture-life-with.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0028-man-walks-in-on-gym-bros-hooking-up-in-the-steam-room-gets-b.jpg</t>
         </is>
       </c>
     </row>
@@ -887,12 +887,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>75 Memes That Perfectly Sum Up The Chaos Of Being Alive Right Now</t>
+          <t>Controlling Parents Hijack Son’s Beach Trip, Call Him Ungrateful When He Cancels The Whole Thing</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0029-75-memes-that-perfectly-sum-up-the-chaos-of-being-alive-righ.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0029-controlling-parents-hijack-sons-beach-trip-call-him-ungratef.jpg</t>
         </is>
       </c>
     </row>
@@ -902,12 +902,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Daily Word Search Game #037 (Jun 24, 2026)</t>
+          <t>Guy Cheats On Wife With A Coworker, Her Kids Methodically Destroy Everything He Built</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0030-daily-word-search-game-037-jun-24-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0030-guy-cheats-on-wife-with-a-coworker-her-kids-methodically-des.jpg</t>
         </is>
       </c>
     </row>
@@ -917,12 +917,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>People Photos From The 2025 Chromatic Awards That Capture The Range Of Culture In Our World (35 Pics)</t>
+          <t>Mom Gets Spoiled All Day On Mother’s Day, Still Finds A Reason To Throw A Massive Tantrum</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0031-people-photos-from-the-2025-chromatic-awards-that-capture-th.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0031-mom-gets-spoiled-all-day-on-mothers-day-still-finds-a-reason.jpg</t>
         </is>
       </c>
     </row>
@@ -932,12 +932,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Rope Jumping Tragedy Continues To Develop As Authorities Arrest Three More Over Disturbing Claims</t>
+          <t>17YO Traumatized With Dad’s Reaction To Her Illness, Ends Up Keeping It A Secret But Drama Ensues</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0032-rope-jumping-tragedy-continues-to-develop-as-authorities-arr.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0032-17yo-traumatized-with-dads-reaction-to-her-illness-ends-up-k.jpg</t>
         </is>
       </c>
     </row>
@@ -947,12 +947,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Animal Behavior Expert Explains 17 Common Things People Get Wrong About Cats</t>
+          <t>35 Times A Friend Did One Thing So Disturbing It Changed How People Saw Them Forever</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0033-animal-behavior-expert-explains-17-common-things-people-get-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0033-35-times-a-friend-did-one-thing-so-disturbing-it-changed-how.jpg</t>
         </is>
       </c>
     </row>
@@ -962,12 +962,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>This Illustrator Reimagined Animals And Places As Human Characters In 22 Playful Artworks</t>
+          <t>Guy Controls Stepdaughter With Ridiculous Rules, Cries Foul As She Finally Cuts Ties For Good</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0034-this-illustrator-reimagined-animals-and-places-as-human-char.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0034-guy-controls-stepdaughter-with-ridiculous-rules-cries-foul-a.jpg</t>
         </is>
       </c>
     </row>
@@ -977,12 +977,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Daily Guess The Famous Person Game #098 (Jun 24, 2026)</t>
+          <t>Employee Asks For A Raise For Years, Boss Learns How Expensive “No” Can Be</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0035-daily-guess-the-famous-person-game-098-jun-24-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0035-employee-asks-for-a-raise-for-years-boss-learns-how-expensiv.jpg</t>
         </is>
       </c>
     </row>
@@ -992,12 +992,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Daily Guess The Timeline Game #092 (Jun 23, 2026)</t>
+          <t>Daily Guess The Timeline Game #086 (Jun 17, 2026)</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0036-daily-guess-the-timeline-game-092-jun-23-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0036-daily-guess-the-timeline-game-086-jun-17-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -1007,12 +1007,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Woman Who Tattooed Both Her Eyes Reveals 10 Ways The Procedure Changed Her Life For The Worse</t>
+          <t>“Is Your Disney IQ Above Average?”: Prove It By Guessing 16 Characters From Their Eyes</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0037-woman-who-tattooed-both-her-eyes-reveals-10-ways-the-procedu.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0037-is-your-disney-iq-above-average-prove-it-by-guessing-16-char.jpg</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>“Descending Into The Abyss”: 60 Liminal Spaces So Deeply Unsettling We’re Sorry In Advance</t>
+          <t>Guy Meets The Wife Of His Ex-Wife’s Affair Partner And Realizes Something</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0038-descending-into-the-abyss-60-liminal-spaces-so-deeply-unsett.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0038-guy-meets-the-wife-of-his-ex-wifes-affair-partner-and-realiz.jpg</t>
         </is>
       </c>
     </row>
@@ -1037,12 +1037,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>38 Clever Comics By This Artist That Joke About Relationships, Technology, And Everyday Anxiety</t>
+          <t>“I Don’t Have A Red Flag”: 27 Questions That Will Probably Prove You Wrong</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0039-38-clever-comics-by-this-artist-that-joke-about-relationship.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0039-i-dont-have-a-red-flag-27-questions-that-will-probably-prove.jpg</t>
         </is>
       </c>
     </row>
@@ -1052,12 +1052,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>“Where Have I Seen That Dress?”: 18 Memorable Outfits For You To Match To The TV Show</t>
+          <t>Millionaire Connected To UK Royals Arrested 9 Years After Jogger Caught On Video pushing Woman In Front Of Bus</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0040-where-have-i-seen-that-dress-18-memorable-outfits-for-you-to.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0040-millionaire-connected-to-uk-royals-arrested-9-years-after-jo.jpg</t>
         </is>
       </c>
     </row>
@@ -1067,12 +1067,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Daily Guess The Country Game #038 (Jun 23, 2026)</t>
+          <t>These 109 Bakers Took Dessert Decorating To An Entirely Different Level (New Pics)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0041-daily-guess-the-country-game-038-jun-23-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0041-these-109-bakers-took-dessert-decorating-to-an-entirely-diff.jpg</t>
         </is>
       </c>
     </row>
@@ -1082,12 +1082,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>85 Tumblr Posts That Deserve To Stay On The Internet Forever (New Pics)</t>
+          <t>A Lifelong Bond Between Siblings Crumbles When Woman Realizes Brother Kept A Major Secret Only From Her</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0042-85-tumblr-posts-that-deserve-to-stay-on-the-internet-forever.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0042-a-lifelong-bond-between-siblings-crumbles-when-woman-realize.jpg</t>
         </is>
       </c>
     </row>
@@ -1097,12 +1097,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>A Longtime New Yorker Cartoonist Captures The Strange Logic Of Everyday Life (24 New Pics)</t>
+          <t>Update In Case Of Imprisoned Woman Who Set Her Male Friend On Fire Over ‘Misogynist’ Comment</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0043-a-longtime-new-yorker-cartoonist-captures-the-strange-logic-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0043-update-in-case-of-imprisoned-woman-who-set-her-male-friend-o.jpg</t>
         </is>
       </c>
     </row>
@@ -1112,12 +1112,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>If You Can Solve All 14 Of These Two-Clue Riddles, You’re More Knowledgeable Than Most</t>
+          <t>“Overstimulating Americanness”: 79 Parts Of US Culture Tourists Weren’t Ready For</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0044-if-you-can-solve-all-14-of-these-two-clue-riddles-youre-more.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0044-overstimulating-americanness-79-parts-of-us-culture-tourists.jpg</t>
         </is>
       </c>
     </row>
@@ -1127,12 +1127,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>A Roman Historian Who Called Christianity Evil Accidentally Wrote The Best Proof That Jesus Existed</t>
+          <t>75 Times Urban Planners Failed To Predict What People Want, And It Resulted In ‘Desire Paths’ Around The City (New Pics)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0045-a-roman-historian-who-called-christianity-evil-accidentally-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0045-75-times-urban-planners-failed-to-predict-what-people-want-a.jpg</t>
         </is>
       </c>
     </row>
@@ -1142,12 +1142,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>If You’re Feeling Down, Here Are 42 Posts That Are Oddly Wholesome</t>
+          <t>Daily Guess The Country Game #032 (Jun 17, 2026)</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0046-if-youre-feeling-down-here-are-42-posts-that-are-oddly-whole.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0046-daily-guess-the-country-game-032-jun-17-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -1157,12 +1157,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Nurses Say These 40 Cases Are The Most Mysterious Things They Saw During Their Career</t>
+          <t>From Public Meltdowns To Strange Confessions, 38 People Share How Their Relationships Ended</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0047-nurses-say-these-40-cases-are-the-most-mysterious-things-the.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0047-from-public-meltdowns-to-strange-confessions-38-people-share.jpg</t>
         </is>
       </c>
     </row>
@@ -1172,12 +1172,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Husband Keeps Saying Wife Has Changed Since Having Kids, She Finally Connects The Dots</t>
+          <t>“I Want People To Feel More Understood”: 30 New Relatable Comics By Krysten Bevilaqua</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0048-husband-keeps-saying-wife-has-changed-since-having-kids-she-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0048-i-want-people-to-feel-more-understood-30-new-relatable-comic.jpg</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1187,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Daily Word Search Game #036 (Jun 23, 2026)</t>
+          <t>“Can You Solve Them All?”: 15 Math Puzzles That Are Trickier Than They First Seem</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0049-daily-word-search-game-036-jun-23-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0049-can-you-solve-them-all-15-math-puzzles-that-are-trickier-tha.jpg</t>
         </is>
       </c>
     </row>
@@ -1202,12 +1202,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Couple Gets Annoyed That SIL’s Cancer Is Overshadowing Their Wedding, The Truth Is Much Worse</t>
+          <t>31 New Comedic Animal Portraits By Alison Friend That Make Pets Look Like Tiny Eccentric Nobles</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0050-couple-gets-annoyed-that-sils-cancer-is-overshadowing-their-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0050-31-new-comedic-animal-portraits-by-alison-friend-that-make-p.jpg</t>
         </is>
       </c>
     </row>
@@ -1217,12 +1217,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Entitled Mom Thinks New Homeowner Owes Her Son An Explanation</t>
+          <t>64 Random Silly Memes That Might Bring A Smile To Anyone Feeling Overwhelmed Today</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0051-entitled-mom-thinks-new-homeowner-owes-her-son-an-explanatio.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0051-64-random-silly-memes-that-might-bring-a-smile-to-anyone-fee.jpg</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1232,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>This Artist Illustrates The Struggles Of An Everyday Girl In These 5 New Comics</t>
+          <t>Daily Word Search Game #030 (Jun 17, 2026)</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0052-this-artist-illustrates-the-struggles-of-an-everyday-girl-in.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0052-daily-word-search-game-030-jun-17-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -1247,12 +1247,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>A History Researcher Reveals 20 Lost Treasures Worth Billions That Have Never Been Found</t>
+          <t>30 Unfiltered Images That Show Real Life Across The Globe By This Street Photographer (New Pics)</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0053-a-history-researcher-reveals-20-lost-treasures-worth-billion.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0053-30-unfiltered-images-that-show-real-life-across-the-globe-by.jpg</t>
         </is>
       </c>
     </row>
@@ -1262,12 +1262,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>These Wawawiwa Comics Are Here To Add Some Wholesome Joy To Your Day (73 New Pics)</t>
+          <t>Rather Than Decorating The Body, I Design Tattoos That Work With It (53 Pics)</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0054-these-wawawiwa-comics-are-here-to-add-some-wholesome-joy-to-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0054-rather-than-decorating-the-body-i-design-tattoos-that-work-w.jpg</t>
         </is>
       </c>
     </row>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>These Memes From “Animals Doing Things” Are Cute, Chaotic, And Very Relatable (40 New Pics)</t>
+          <t>103 Tattoo Fails That Are Impossible To Ignore (New Pics)</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0055-these-memes-from-animals-doing-things-are-cute-chaotic-and-v.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0055-103-tattoo-fails-that-are-impossible-to-ignore-new-pics.jpg</t>
         </is>
       </c>
     </row>
@@ -1292,12 +1292,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>95 Posts That Taught People Something They Never Knew They Needed To Know</t>
+          <t>“It Was A Cult”: 49 Times People Realized That Something Was Very Wrong And They Needed To Leave</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0056-95-posts-that-taught-people-something-they-never-knew-they-n.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0056-it-was-a-cult-49-times-people-realized-that-something-was-ve.jpg</t>
         </is>
       </c>
     </row>
@@ -1307,12 +1307,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>54 Hilarious Signs Found In The Wild That Prove Park Rangers Have The Best Sense Of Humor</t>
+          <t>Bride Couldn’t Believe What MIL Did At The Wedding, Neither Could The Guests</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0057-54-hilarious-signs-found-in-the-wild-that-prove-park-rangers.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0057-bride-couldnt-believe-what-mil-did-at-the-wedding-neither-co.jpg</t>
         </is>
       </c>
     </row>
@@ -1322,12 +1322,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Parents Think They Can Still Control Their Adult Daughter, Things Don’t Go As Planned</t>
+          <t>82 Incredible Historical Finds That Left People Staring In Disbelief (New Pics)</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0058-parents-think-they-can-still-control-their-adult-daughter-th.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0058-82-incredible-historical-finds-that-left-people-staring-in-d.jpg</t>
         </is>
       </c>
     </row>
@@ -1337,12 +1337,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>107 Brutal Roasts The Victims Probably Still Think About</t>
+          <t>Daily Guess The Famous Person Game #091 (Jun 17, 2026)</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0059-107-brutal-roasts-the-victims-probably-still-think-about.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0059-daily-guess-the-famous-person-game-091-jun-17-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -1352,12 +1352,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>“It’s Super Meaningful”: 65 People Share The Stories Behind Their Most Cherished Tattoos</t>
+          <t>56 Women Share The Comments They Received About Their Bodies That They Didn’t See Coming</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0060-its-super-meaningful-65-people-share-the-stories-behind-thei.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0060-56-women-share-the-comments-they-received-about-their-bodies.jpg</t>
         </is>
       </c>
     </row>
@@ -1367,12 +1367,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>52 Pics That Prove Slavic People Operate On A Wavelength The Rest Of Us Can’t Access</t>
+          <t>Conservative Law Allows Pharmacists To Deny Service, But One 85-Year-Old’s Epic Response Leaves Them Stunned</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0061-52-pics-that-prove-slavic-people-operate-on-a-wavelength-the.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0061-conservative-law-allows-pharmacists-to-deny-service-but-one-.jpg</t>
         </is>
       </c>
     </row>
@@ -1382,12 +1382,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Mom Of Girls Harassed By “Male Karen” In Viral Restroom Video Breaks Silence With Scathing Post Against Dad</t>
+          <t>Exhausted Wife Works Two Jobs While Unemployed Husband Lives In Digital Reality Thinking He’s Productive</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0062-mom-of-girls-harassed-by-male-karen-in-viral-restroom-video-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0062-exhausted-wife-works-two-jobs-while-unemployed-husband-lives.jpg</t>
         </is>
       </c>
     </row>
@@ -1397,12 +1397,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>73 Random Facts That Might Make People Go: “Why On Earth Do You Know That?”</t>
+          <t>42 Experiences With The Youngest Generation That Make People Feel The World Is Doomed</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0063-73-random-facts-that-might-make-people-go-why-on-earth-do-yo.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0063-42-experiences-with-the-youngest-generation-that-make-people.jpg</t>
         </is>
       </c>
     </row>
@@ -1412,12 +1412,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>49 Things People Said Really Hurt Them Despite Their High Pain Tolerance</t>
+          <t>Dad Spent All His Money On Stepdaughter While Watching Bio Kids Suffer, Son Devastated By The Truth</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0064-49-things-people-said-really-hurt-them-despite-their-high-pa.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0064-dad-spent-all-his-money-on-stepdaughter-while-watching-bio-k.jpg</t>
         </is>
       </c>
     </row>
@@ -1427,12 +1427,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Woman Confused Why MIL Can’t Wear White To Her Wedding, Groom Makes An Update And Shares What Happened</t>
+          <t>Toxic Boss Forced To Close Business After Insulting Top Performer, Ends Up Having His Clients Stolen</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0065-woman-confused-why-mil-cant-wear-white-to-her-wedding-groom-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0065-toxic-boss-forced-to-close-business-after-insulting-top-perf.jpg</t>
         </is>
       </c>
     </row>
@@ -1442,12 +1442,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>This Artist’s Watercolor Cat Paintings Are Full Of Personality And Charm (45 Pics)</t>
+          <t>Delulu Mom Wants A Perfect Blended Family, Throws A Hissy Fit When Kids Reject Her Ideology</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0066-this-artists-watercolor-cat-paintings-are-full-of-personalit.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0066-delulu-mom-wants-a-perfect-blended-family-throws-a-hissy-fit.jpg</t>
         </is>
       </c>
     </row>
@@ -1457,12 +1457,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>22 Prime Day Deals So Good We Actually Gasped A Little When We Saw The Prices</t>
+          <t>Postpartum Wife’s 1000 Tinder Matches Shock Hubby, But The Truth Shatters Him More</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0067-22-prime-day-deals-so-good-we-actually-gasped-a-little-when-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0067-postpartum-wifes-1000-tinder-matches-shock-hubby-but-the-tru.jpg</t>
         </is>
       </c>
     </row>
@@ -1472,12 +1472,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>“Paint The Stairs Pink”: 44 Silly Solutions To Really Serious Issues</t>
+          <t>Woman Can’t Figure Out Why Her Wedding News Falls Flat, Best Friend Knows The Uncomfortable Truth</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0068-paint-the-stairs-pink-44-silly-solutions-to-really-serious-i.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0068-woman-cant-figure-out-why-her-wedding-news-falls-flat-best-f.jpg</t>
         </is>
       </c>
     </row>
@@ -1487,12 +1487,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>These 27 General Knowledge Questions Start Easy, And End Surprisingly Hard</t>
+          <t>Family Bows To Demanding MIL’s Every Wish, Woman Becomes The First To Stand Up To Her</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0069-these-27-general-knowledge-questions-start-easy-and-end-surp.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0069-family-bows-to-demanding-mils-every-wish-woman-becomes-the-f.jpg</t>
         </is>
       </c>
     </row>
@@ -1502,12 +1502,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Daily Guess The Famous Person Game #097 (Jun 23, 2026)</t>
+          <t>Unhinged Woman Sparks Drama With Her Racism All Because Her Crush Drew Her Bestie’s Portrait</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0070-daily-guess-the-famous-person-game-097-jun-23-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0070-unhinged-woman-sparks-drama-with-her-racism-all-because-her-.jpg</t>
         </is>
       </c>
     </row>
@@ -1517,12 +1517,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Woman Loses It After BF Reveals Stepsis Was His Ex And That He Wants Her As Bridesmaid</t>
+          <t>Cranky Neighbor Sparks Property Feud, Creates Huge Mess For Himself Instead</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0071-woman-loses-it-after-bf-reveals-stepsis-was-his-ex-and-that-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0071-cranky-neighbor-sparks-property-feud-creates-huge-mess-for-h.jpg</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Student Baffled Over Her Parents’ Unexpected Hostility As They Give Her Room To Jobless Brother</t>
+          <t>“Your Body Will Simply Give Up”: 38 Human Body Facts That Might Make You Scared To Be Alive</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0072-student-baffled-over-her-parents-unexpected-hostility-as-the.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0072-your-body-will-simply-give-up-38-human-body-facts-that-might.jpg</t>
         </is>
       </c>
     </row>
@@ -1547,12 +1547,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Dad And His Friend Joke About Daughters Being Difficult, One Remark From His Teen Changes The Mood</t>
+          <t>Daily Guess The Timeline Game #085 (Jun 16, 2026)</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0073-dad-and-his-friend-joke-about-daughters-being-difficult-one-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0073-daily-guess-the-timeline-game-085-jun-16-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -1562,12 +1562,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Woman Disinvited From Hubs’ Bestie’s Destination Wedding Last-Minute, Hubs Sees Red And RSVPs No</t>
+          <t>Mom Thinks Everyone Else Is Overreacting To Daughter’s Behavior, Commenters Disagree</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0074-woman-disinvited-from-hubs-besties-destination-wedding-last-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0074-mom-thinks-everyone-else-is-overreacting-to-daughters-behavi.jpg</t>
         </is>
       </c>
     </row>
@@ -1577,12 +1577,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Wife Asks To Hang Out With Guy She Opened The Marriage For, Her Husband Has Finally Had Enough</t>
+          <t>“She Refused To Speak To The Staff”: 35 Celebrity Encounters That Were A Lot To Witness</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0075-wife-asks-to-hang-out-with-guy-she-opened-the-marriage-for-h.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0075-she-refused-to-speak-to-the-staff-35-celebrity-encounters-th.jpg</t>
         </is>
       </c>
     </row>
@@ -1592,12 +1592,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Manipulative Mom Tried To Sneak Her Son Onto A Vacation, It Blows Up Hard On Her Face</t>
+          <t>Woman Survives A Workplace Emergency, Then Finds Herself In Even More Trouble</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0076-manipulative-mom-tried-to-sneak-her-son-onto-a-vacation-it-b.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0076-woman-survives-a-workplace-emergency-then-finds-herself-in-e.jpg</t>
         </is>
       </c>
     </row>
@@ -1607,12 +1607,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Birthday Woman Chooses Thai Restaurant For Dinner, Then Gets Cut Out Of Her Own Party</t>
+          <t>19 Celebrities Showed Up To Watch UFC At The White House, And The Guest List Is A Lot To Process</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0077-birthday-woman-chooses-thai-restaurant-for-dinner-then-gets-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0077-19-celebrities-showed-up-to-watch-ufc-at-the-white-house-and.jpg</t>
         </is>
       </c>
     </row>
@@ -1622,12 +1622,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Toxic Friend Frames Woman And Steals Her Blind Date, Gets What She Deserved The Very Next Day</t>
+          <t>Passenger Tormented By Racist Woman On Flight Gets An Upgrade, She Gets Shut Down By The Crew</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0078-toxic-friend-frames-woman-and-steals-her-blind-date-gets-wha.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0078-passenger-tormented-by-racist-woman-on-flight-gets-an-upgrad.jpg</t>
         </is>
       </c>
     </row>
@@ -1637,12 +1637,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Daily Guess The Timeline Game #091 (Jun 22, 2026)</t>
+          <t>21 Mind-Bending Dilemmas That’ll Challenge Your Morals: Vote Now &amp; See Where You Stand</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0079-daily-guess-the-timeline-game-091-jun-22-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0079-21-mind-bending-dilemmas-thatll-challenge-your-morals-vote-n.jpg</t>
         </is>
       </c>
     </row>
@@ -1652,12 +1652,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>57 Times People Laughed Without Context And Immediately Regretted It</t>
+          <t>53 Toxic Friends Who Hurt People In Ways They Never Saw Coming</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0080-57-times-people-laughed-without-context-and-immediately-regr.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0080-53-toxic-friends-who-hurt-people-in-ways-they-never-saw-comi.jpg</t>
         </is>
       </c>
     </row>
@@ -1667,12 +1667,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>53 Airport Photos So Ridiculous They Might Make Travelers Miss Their Flights From Laughing</t>
+          <t>Children Of Karen Parents Are Sharing Their Wildest Stories, And They’re Brutal</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0081-53-airport-photos-so-ridiculous-they-might-make-travelers-mi.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0081-children-of-karen-parents-are-sharing-their-wildest-stories-.jpg</t>
         </is>
       </c>
     </row>
@@ -1682,12 +1682,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>15 Modern Adulting Questions Every Grown-Up Should Be Able To Answer – Test Yourself</t>
+          <t>Trauma Bonding: Signs, Stages, and How to Break Free</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0082-15-modern-adulting-questions-every-grown-up-should-be-able-t.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0082-trauma-bonding-signs-stages-and-how-to-break-free.jpg</t>
         </is>
       </c>
     </row>
@@ -1697,12 +1697,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Daily Guess The Country Game #037 (Jun 22, 2026)</t>
+          <t>Narcissistic Guy Refuses To Pay Spousal Support And Takes Ex To Court, Ends Up Paying With 401k</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0083-daily-guess-the-country-game-037-jun-22-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0083-narcissistic-guy-refuses-to-pay-spousal-support-and-takes-ex.jpg</t>
         </is>
       </c>
     </row>
@@ -1712,12 +1712,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>65 New Sarcasm-Filled Comics By The Artist Steve Nelson</t>
+          <t>I Illustrate The Hilarious Reality Of A Rescue Dog And A Cat Living Together (25 New Comics)</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0084-65-new-sarcasm-filled-comics-by-the-artist-steve-nelson.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0084-i-illustrate-the-hilarious-reality-of-a-rescue-dog-and-a-cat.jpg</t>
         </is>
       </c>
     </row>
@@ -1727,12 +1727,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>64 Times People Asked Their Partner To Stop Doing Something Gross, And Failed</t>
+          <t>Daily Guess The Country Game #031 (Jun 16, 2026)</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0085-64-times-people-asked-their-partner-to-stop-doing-something-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0085-daily-guess-the-country-game-031-jun-16-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -1742,12 +1742,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Guy Has Suspicions Over Daughter Not Being His, Turns Out It’s Way Worse Than He Could Have Guessed</t>
+          <t>This Photographer Captured 42 Dreamlike Images Of Antarctica</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0086-guy-has-suspicions-over-daughter-not-being-his-turns-out-its.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0086-this-photographer-captured-42-dreamlike-images-of-antarctica.jpg</t>
         </is>
       </c>
     </row>
@@ -1757,12 +1757,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>74 Electronics Fails So Bad They Basically Wrote Their Own Eulogy</t>
+          <t>39 Captivating Travel Photos From The 2025 Chromatic Awards That Show How Diverse The World Is</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0087-74-electronics-fails-so-bad-they-basically-wrote-their-own-e.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0087-39-captivating-travel-photos-from-the-2025-chromatic-awards-.jpg</t>
         </is>
       </c>
     </row>
@@ -1772,12 +1772,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>18 Human Habits That Confuse Dogs The Most, According To An Animal Behaviorist</t>
+          <t>“Can You Still Solve Basic Equations?”: Ace This 20-Question Math Quiz And Reveal The Truth</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0088-18-human-habits-that-confuse-dogs-the-most-according-to-an-a.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0088-can-you-still-solve-basic-equations-ace-this-20-question-mat.jpg</t>
         </is>
       </c>
     </row>
@@ -1787,12 +1787,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Name All 22 World Capitals From Two Clues Each – Prove Your Geography Knowledge</t>
+          <t>This Page Shared 26 Heartwarming Animal Moments From Around The World (New Pics)</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0089-name-all-22-world-capitals-from-two-clues-each-prove-your-ge.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0089-this-page-shared-26-heartwarming-animal-moments-from-around-.jpg</t>
         </is>
       </c>
     </row>
@@ -1802,12 +1802,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>63 Absolutely Atrocious Clothing Design Fails That Might Make You Giggle</t>
+          <t>25 Remarkable Dog Rescue Transformations Shared By NIRA That Show The Power Of A Second Chance</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0090-63-absolutely-atrocious-clothing-design-fails-that-might-mak.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0090-25-remarkable-dog-rescue-transformations-shared-by-nira-that.jpg</t>
         </is>
       </c>
     </row>
@@ -1817,12 +1817,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Artist Shares 57 New Comics About Ferrets, Pets, And Everyday Absurdities</t>
+          <t>Daily Word Search Game #029 (Jun 16, 2026)</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0091-artist-shares-57-new-comics-about-ferrets-pets-and-everyday-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0091-daily-word-search-game-029-jun-16-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -1830,8 +1830,16 @@
       <c r="A93" t="n">
         <v>92</v>
       </c>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr"/>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>23 Hilarious Father’s Day Gifts For The Dad Whose Sense Of Humor Is The Best Thing He Passed Down</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0092-23-hilarious-fathers-day-gifts-for-the-dad-whose-sense-of-hu.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -1839,12 +1847,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Daily Word Search Game #035 (Jun 22, 2026)</t>
+          <t>30 New Comics By Brian Gordon Showcasing The Funny Side Of Parenting</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0093-daily-word-search-game-035-jun-22-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0093-30-new-comics-by-brian-gordon-showcasing-the-funny-side-of-p.jpg</t>
         </is>
       </c>
     </row>
@@ -1854,12 +1862,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>“Bride Of Chucky”: Evil MIL Takes Twisted Joke A Step Too Far, Leaving Wedding Guests Horrified</t>
+          <t>Emily Ratajkowski Faces Backlash Over Essay About Single Motherhood Accompanied By Bizarre Breastfeeding Photo</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0094-bride-of-chucky-evil-mil-takes-twisted-joke-a-step-too-far-l.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0094-emily-ratajkowski-faces-backlash-over-essay-about-single-mot.jpg</t>
         </is>
       </c>
     </row>
@@ -1869,12 +1877,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Woman Loses Husband And Best Friend To An Affair, Gets The Last Laugh Years Later</t>
+          <t>67 Brutally Honest Posts From Millennials On Social Media (New Pics)</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0095-woman-loses-husband-and-best-friend-to-an-affair-gets-the-la.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0095-67-brutally-honest-posts-from-millennials-on-social-media-ne.jpg</t>
         </is>
       </c>
     </row>
@@ -1884,12 +1892,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>84 Tragic Hair Accidents That Should Never Have Seen The Light Of Day (New Pics)</t>
+          <t>63 Awkward Texts That Are So Bad It’s Funny (New Pics)</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0096-84-tragic-hair-accidents-that-should-never-have-seen-the-lig.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0096-63-awkward-texts-that-are-so-bad-its-funny-new-pics.jpg</t>
         </is>
       </c>
     </row>
@@ -1899,12 +1907,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>35 Cases So Bizarre People Still Argue About Them Today</t>
+          <t>“Unsure About Dinosaurs”: 50 People Who Dated Morons Reveal Their Dumbest Beliefs</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0097-35-cases-so-bizarre-people-still-argue-about-them-today.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0097-unsure-about-dinosaurs-50-people-who-dated-morons-reveal-the.jpg</t>
         </is>
       </c>
     </row>
@@ -1914,12 +1922,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Guy Tries To Control What Neighbor Wears Outside, Doesn’t Get The Response He Wanted</t>
+          <t>This Instagram Account Shares Hilarious Design Fails, Here Are 91 Of The Best (New Pics)</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0098-guy-tries-to-control-what-neighbor-wears-outside-doesnt-get-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0098-this-instagram-account-shares-hilarious-design-fails-here-ar.jpg</t>
         </is>
       </c>
     </row>
@@ -1929,12 +1937,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>“Wake My Son Up For School”: 65 Entitled Messages That Left Teachers Speechless</t>
+          <t>Spiteful Grandma Spills Decades-Old Secret In Most Brutal Way Possible And Faces Immediate Family Exile</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0099-wake-my-son-up-for-school-65-entitled-messages-that-left-tea.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0099-spiteful-grandma-spills-decades-old-secret-in-most-brutal-wa.jpg</t>
         </is>
       </c>
     </row>
@@ -1944,12 +1952,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Daily Guess The Famous Person Game #096 (Jun 22, 2026)</t>
+          <t>This Page Shared 65 Irresistible Pics Of Baby Animals And Their Moms</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0100-daily-guess-the-famous-person-game-096-jun-22-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0100-this-page-shared-65-irresistible-pics-of-baby-animals-and-th.jpg</t>
         </is>
       </c>
     </row>
@@ -1959,12 +1967,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>56 Secrets People In Long-Term Relationships Are Keeping From Their Partners</t>
+          <t>Daily Guess The Famous Person Game #090 (Jun 16, 2026)</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0101-56-secrets-people-in-long-term-relationships-are-keeping-fro.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0101-daily-guess-the-famous-person-game-090-jun-16-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -1974,12 +1982,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>“How Academic Are You?”: 25 Smart English Words That Only Advanced Speakers Know</t>
+          <t>We Prepared 26 Pop Culture Questions From A To Z – Anything Above 22 Is An Excellent Score</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0102-how-academic-are-you-25-smart-english-words-that-only-advanc.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0102-we-prepared-26-pop-culture-questions-from-a-to-z-anything-ab.jpg</t>
         </is>
       </c>
     </row>
@@ -1989,12 +1997,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>16 Prime Day Deals That Started Early And Are Honestly Too Good To Just Scroll Past</t>
+          <t>30 Times Folks Online Were Disturbed By The People Their Friends Were Dating</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0103-16-prime-day-deals-that-started-early-and-are-honestly-too-g.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0103-30-times-folks-online-were-disturbed-by-the-people-their-fri.jpg</t>
         </is>
       </c>
     </row>
@@ -2004,12 +2012,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Bride Lies About Food At Her Wedding To Prove A Point But Only Gets Coworker’s Child Hospitalized</t>
+          <t>71 Times People Thought They Took Normal Photos Until They Turned Into Hilarious ‘When You See It’ Moments (New Pics)</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0104-bride-lies-about-food-at-her-wedding-to-prove-a-point-but-on.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0104-71-times-people-thought-they-took-normal-photos-until-they-t.jpg</t>
         </is>
       </c>
     </row>
@@ -2019,12 +2027,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>71 Posts That Gave People An Unexpected Existential Crisis About Their Age (New Pics)</t>
+          <t>19YO Gets Dismissed By Know-It-All Nurse, Returns A Week Later With A Huge Infection Instead</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0105-71-posts-that-gave-people-an-unexpected-existential-crisis-a.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0105-19yo-gets-dismissed-by-know-it-all-nurse-returns-a-week-late.jpg</t>
         </is>
       </c>
     </row>
@@ -2034,12 +2042,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>“It Didn’t Work”: 43 Stories About What It’s Really Like To Live In A Polygamist Household</t>
+          <t>Aunt Tired Of Playing Emergency Contact For 5YO In Constant Trouble, Demands Parents Face Reality</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0106-it-didnt-work-43-stories-about-what-its-really-like-to-live-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0106-aunt-tired-of-playing-emergency-contact-for-5yo-in-constant-.jpg</t>
         </is>
       </c>
     </row>
@@ -2049,12 +2057,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>People Are Sharing The Most Infuriating But Also Hilarious Food Delivery Driver Fails</t>
+          <t>VIP Passenger Picks Drinking Over Taking Care Of Her Kids, Pilot Ends Up Teaching Her A Lesson</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0107-people-are-sharing-the-most-infuriating-but-also-hilarious-f.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0107-vip-passenger-picks-drinking-over-taking-care-of-her-kids-pi.jpg</t>
         </is>
       </c>
     </row>
@@ -2064,12 +2072,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>“Am I The Jerk For Telling My Dad I Don’t Care About The Kids He Replaced Me With?”</t>
+          <t>Couple Are Warned About Nightmare Neighbor, Move In Across The Road Anyway, Regret It Immediately</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0108-am-i-the-jerk-for-telling-my-dad-i-dont-care-about-the-kids-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0108-couple-are-warned-about-nightmare-neighbor-move-in-across-th.jpg</t>
         </is>
       </c>
     </row>
@@ -2079,12 +2087,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Family Tries To Challenge Grandma’s Will At Her Funeral, One Man’s Speech Changes Everything</t>
+          <t>Vicious Aunt Berates “Unladylike” Niece, Doesn’t Realize She’s Saying Goodbye To Her Own Cash Flow</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0109-family-tries-to-challenge-grandmas-will-at-her-funeral-one-m.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0109-vicious-aunt-berates-unladylike-niece-doesnt-realize-shes-sa.jpg</t>
         </is>
       </c>
     </row>
@@ -2094,12 +2102,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Parents Laugh When Son Says They Always Choose Adopted Kid, He Returns The Favor By Ditching Them</t>
+          <t>Mom Lets Stepkids Make Daughter Miserable For Years, Suddenly Wants A Second Chance When She’s Gone</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0110-parents-laugh-when-son-says-they-always-choose-adopted-kid-h.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0110-mom-lets-stepkids-make-daughter-miserable-for-years-suddenly.jpg</t>
         </is>
       </c>
     </row>
@@ -2109,12 +2117,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Attention-Hungry Blogger Exposes Her Family For Clicks, It Blows Up In Her Face</t>
+          <t>49 People With Jobs So Strange Most People Don’t Know They Exist</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0111-attention-hungry-blogger-exposes-her-family-for-clicks-it-bl.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0111-49-people-with-jobs-so-strange-most-people-dont-know-they-ex.jpg</t>
         </is>
       </c>
     </row>
@@ -2124,12 +2132,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>35 Celebrity Scandals That Were So Ridiculous That We’re Still Shocked They Even Happened</t>
+          <t>73 Cursed Images From This Weird Corner Of The Internet (New Pics)</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0112-35-celebrity-scandals-that-were-so-ridiculous-that-were-stil.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0112-73-cursed-images-from-this-weird-corner-of-the-internet-new-.jpg</t>
         </is>
       </c>
     </row>
@@ -2139,12 +2147,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Woman Watches Her Sisterly Bond With Adopted Sis Crumble After Disturbing Wedding Debacle</t>
+          <t>Barron Trump’s UFC Appearance Fuels Concern And Wild Speculation About His Changed Look: “Absolutely Miserable”</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0113-woman-watches-her-sisterly-bond-with-adopted-sis-crumble-aft.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0113-barron-trumps-ufc-appearance-fuels-concern-and-wild-speculat.jpg</t>
         </is>
       </c>
     </row>
@@ -2154,12 +2162,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>19 World Cup Stars So Handsome, Fans Can’t Stop Talking About Them</t>
+          <t>50 Funny Cat Memes That Prove Life Is Better When Cats Are Being Weird</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0114-19-world-cup-stars-so-handsome-fans-cant-stop-talking-about-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0114-50-funny-cat-memes-that-prove-life-is-better-when-cats-are-b.jpg</t>
         </is>
       </c>
     </row>
@@ -2169,12 +2177,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Daily Guess The Timeline Game #090 (Jun 21, 2026)</t>
+          <t>“Never Expected Me To Turn Her Own Logic Against Her”: Woman Shocks MIL With A Savage Comeback</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0115-daily-guess-the-timeline-game-090-jun-21-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0115-never-expected-me-to-turn-her-own-logic-against-her-woman-sh.jpg</t>
         </is>
       </c>
     </row>
@@ -2184,12 +2192,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>This Scottish X Account Went Viral For Explaining US Slang, Here Are Its 13 Best Posts</t>
+          <t>“If Your Arm Is Gone, It’s A Jaguar”: 73 Animal Facts That Sent Us Down A Rabbit Hole For Hours</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0116-this-scottish-x-account-went-viral-for-explaining-us-slang-h.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0116-if-your-arm-is-gone-its-a-jaguar-73-animal-facts-that-sent-u.jpg</t>
         </is>
       </c>
     </row>
@@ -2199,12 +2207,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>97 “Epic Top Comments” That Are Way More Entertaining Than The Posts They’re On</t>
+          <t>‘Karen’ Proves That Some Parents Need To Snap Back To Reality After She Attacks Disabled Person</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0117-97-epic-top-comments-that-are-way-more-entertaining-than-the.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0117-karen-proves-that-some-parents-need-to-snap-back-to-reality-.jpg</t>
         </is>
       </c>
     </row>
@@ -2214,12 +2222,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>These 53 Memes Are So Funny They Might Make You Question Your Sanity In The Best Way</t>
+          <t>Daily Guess The Timeline Game #084 (Jun 15, 2026)</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0118-these-53-memes-are-so-funny-they-might-make-you-question-you.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0118-daily-guess-the-timeline-game-084-jun-15-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -2229,12 +2237,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>“Ancient Macedonian Gold”: 71 Authentic Historical Finds That Might Feel Like Time Travel</t>
+          <t>Woman Shocked That She Might Be “Stealing Friend’s Boyfriend,” The Truth Is More Bizarre Than She Expected</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0119-ancient-macedonian-gold-71-authentic-historical-finds-that-m.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0119-woman-shocked-that-she-might-be-stealing-friends-boyfriend-t.jpg</t>
         </is>
       </c>
     </row>
@@ -2244,12 +2252,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>62 Hilarious Dads Who Were Clearly Born For The Role (New Pics)</t>
+          <t>33 Folks Who Believed Their Friends Were Just “Nice Peeps,” Until Some Discovery Proved The Opposite</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0120-62-hilarious-dads-who-were-clearly-born-for-the-role-new-pic.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0120-33-folks-who-believed-their-friends-were-just-nice-peeps-unt.jpg</t>
         </is>
       </c>
     </row>
@@ -2259,12 +2267,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>77 Cringy And Sad Moments That Will Forever Live As Screenshots On The Internet</t>
+          <t>“Never Came Back To School”: 51 Times The Class Clown Took It Too Far And Faced The Consequences</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0121-77-cringy-and-sad-moments-that-will-forever-live-as-screensh.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0121-never-came-back-to-school-51-times-the-class-clown-took-it-t.jpg</t>
         </is>
       </c>
     </row>
@@ -2274,12 +2282,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>“It Breaks My Heart”: 32 Popular Kids Who Threw Everything Away</t>
+          <t>Only True Music Fans Can Name All 25 Iconic Titles From A Blurry Image</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0122-it-breaks-my-heart-32-popular-kids-who-threw-everything-away.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0122-only-true-music-fans-can-name-all-25-iconic-titles-from-a-bl.jpg</t>
         </is>
       </c>
     </row>
@@ -2289,12 +2297,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>69 Coincidences So Crazy People Still Can’t Wrap Their Heads Around Them</t>
+          <t>We Highly Doubt You Can Beat The Average U.S. Student – Prove Us Wrong In 18 Questions</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0123-69-coincidences-so-crazy-people-still-cant-wrap-their-heads-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0123-we-highly-doubt-you-can-beat-the-average-us-student-prove-us.jpg</t>
         </is>
       </c>
     </row>
@@ -2304,12 +2312,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>75 Creepy Facts And Horror Stories People Wish They Never Learned</t>
+          <t>Woman Finds Out She’s No Longer Invited To Friend’s Wedding, Karma Hits Right Before The Big Day</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0124-75-creepy-facts-and-horror-stories-people-wish-they-never-le.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0124-woman-finds-out-shes-no-longer-invited-to-friends-wedding-ka.jpg</t>
         </is>
       </c>
     </row>
@@ -2319,12 +2327,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>24 Wholesome Posts From The “One Night I Was Bored In Bed” Trend</t>
+          <t>57 Hilariously Random Screenshots That Were Too Funny Not To Share (New Pics)</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0125-24-wholesome-posts-from-the-one-night-i-was-bored-in-bed-tre.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0125-57-hilariously-random-screenshots-that-were-too-funny-not-to.jpg</t>
         </is>
       </c>
     </row>
@@ -2334,12 +2342,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>“Can You Actually Decide?”: Vote On 17 ‘Would You Rather’ Questions From Films, TV &amp; Books</t>
+          <t>“Is It Tokyo Or Seoul?”: Challenge Your Memory Of The Capitals With 18 Borderless Maps</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0126-can-you-actually-decide-vote-on-17-would-you-rather-question.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0126-is-it-tokyo-or-seoul-challenge-your-memory-of-the-capitals-w.jpg</t>
         </is>
       </c>
     </row>
@@ -2349,12 +2357,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Man Is So Glad He’s Escaping Controlling Fiancée After Finally Checking Their Joint Bank Account</t>
+          <t>Daily Guess The Country Game #030 (Jun 15, 2026)</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0127-man-is-so-glad-hes-escaping-controlling-fiancee-after-finall.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0127-daily-guess-the-country-game-030-jun-15-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -2364,12 +2372,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Daily Guess The Country Game #036 (Jun 21, 2026)</t>
+          <t>If You Like Dry Humor, Here Are 58 New One-Panel Comics By Graham Annable To Enjoy</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0128-daily-guess-the-country-game-036-jun-21-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0128-if-you-like-dry-humor-here-are-58-new-one-panel-comics-by-gr.jpg</t>
         </is>
       </c>
     </row>
@@ -2379,12 +2387,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Daily Word Search Game #034 (Jun 21, 2026)</t>
+          <t>43 Underwater Oil Paintings By This Artist, So Beautiful They Feel Like Memories In Motion</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0129-daily-word-search-game-034-jun-21-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0129-43-underwater-oil-paintings-by-this-artist-so-beautiful-they.jpg</t>
         </is>
       </c>
     </row>
@@ -2394,12 +2402,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Daily Guess The Famous Person Game #095 (Jun 21, 2026)</t>
+          <t>Daily Word Search Game #028 (Jun 15, 2026)</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0130-daily-guess-the-famous-person-game-095-jun-21-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0130-daily-word-search-game-028-jun-15-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -2409,12 +2417,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Daily Guess The Timeline Game #089 (Jun 20, 2026)</t>
+          <t>‘House Of The Dragon’ Season 3 Cast Guide: Every New and Returning Character</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0131-daily-guess-the-timeline-game-089-jun-20-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0131-house-of-the-dragon-season-3-cast-guide-every-new-and-return.jpg</t>
         </is>
       </c>
     </row>
@@ -2424,12 +2432,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>If You Need To Take A Mental Break, These 55 Posts Should Help You Decompress Like A Hot Bath</t>
+          <t>55 Memes Shared By The ‘Ancient Cringe’ Page That Turn Historical Art Into Relatable Comedy</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0132-if-you-need-to-take-a-mental-break-these-55-posts-should-hel.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0132-55-memes-shared-by-the-ancient-cringe-page-that-turn-histori.jpg</t>
         </is>
       </c>
     </row>
@@ -2439,12 +2447,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>“There Was No Grass In Dinosaur Times”: 52 Facts That You Might Not Believe Are Actually True</t>
+          <t>30 Futuristic Chrome Tattoos By This Artist That Look Like They Were Imported From The Future</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0133-there-was-no-grass-in-dinosaur-times-52-facts-that-you-might.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0133-30-futuristic-chrome-tattoos-by-this-artist-that-look-like-t.jpg</t>
         </is>
       </c>
     </row>
@@ -2454,12 +2462,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>56 ER Patients Share The Mistakes That Sent Them To The Hospital</t>
+          <t>Daily Guess The Famous Person Game #089 (Jun 15, 2026)</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0134-56-er-patients-share-the-mistakes-that-sent-them-to-the-hosp.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0134-daily-guess-the-famous-person-game-089-jun-15-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -2469,12 +2477,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>“Future Tech”: 33 Things People Are Working On Now That Might Change Everything</t>
+          <t>“What Is Something That Is Highly Likely To Happen In The Next 10 Years That Everyone Is Completely Ignoring?” (67 Answers)</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0135-future-tech-33-things-people-are-working-on-now-that-might-c.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0135-what-is-something-that-is-highly-likely-to-happen-in-the-nex.jpg</t>
         </is>
       </c>
     </row>
@@ -2484,12 +2492,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>71 History Posts That Sent People Down Unexpected Rabbit Holes</t>
+          <t>We All Make Mistakes, But These 60 Huge Fails Hurt To Laugh At (New Pics)</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0136-71-history-posts-that-sent-people-down-unexpected-rabbit-hol.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0136-we-all-make-mistakes-but-these-60-huge-fails-hurt-to-laugh-a.jpg</t>
         </is>
       </c>
     </row>
@@ -2499,12 +2507,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>The Office Struggle Is Real And People Cope By Creating These 77 Hilarious Memes (New Pics)</t>
+          <t>Regretful Husband Deserts His Marriage For A Younger Fantasy, And Now He Can’t Handle The Reality</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0137-the-office-struggle-is-real-and-people-cope-by-creating-thes.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0137-regretful-husband-deserts-his-marriage-for-a-younger-fantasy.jpg</t>
         </is>
       </c>
     </row>
@@ -2514,12 +2522,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>97 Amazing Facts About Our World To Keep You Busy For A Few Minutes</t>
+          <t>New Mom Shocked After Half-Sis Who Struggles With Infertility Said Newborn Was Hers</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0138-97-amazing-facts-about-our-world-to-keep-you-busy-for-a-few-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0138-new-mom-shocked-after-half-sis-who-struggles-with-infertilit.jpg</t>
         </is>
       </c>
     </row>
@@ -2529,12 +2537,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Thousands Of People Love This Page’s Random Sense Of Humor, Here Are 67 Of Its Best Posts</t>
+          <t>20 Harsh Reality Checks From The “Awful Everything” Group That Might Change Your View On Things (New Pics)</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0139-thousands-of-people-love-this-pages-random-sense-of-humor-he.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0139-20-harsh-reality-checks-from-the-awful-everything-group-that.jpg</t>
         </is>
       </c>
     </row>
@@ -2544,12 +2552,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>56 Of The Funniest Pop Culture Posts You Can Pass Around For Instant Good Vibes</t>
+          <t>41 Satisfying Petty Revenge Stories Where Cheaters Got What They Deserved</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0140-56-of-the-funniest-pop-culture-posts-you-can-pass-around-for.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0140-41-satisfying-petty-revenge-stories-where-cheaters-got-what-.jpg</t>
         </is>
       </c>
     </row>
@@ -2559,12 +2567,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Couple Has To Change Locks Over MIL’s Behavior, She Refuses To Back Down</t>
+          <t>“AITA For Telling My Family The Real Reason My Mother And I Are Not Attending My Sister’s Wedding?”</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0141-couple-has-to-change-locks-over-mils-behavior-she-refuses-to.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0141-aita-for-telling-my-family-the-real-reason-my-mother-and-i-a.jpg</t>
         </is>
       </c>
     </row>
@@ -2574,12 +2582,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Wife Learns Husband Orchestrated Their Relationship After Shocking Discovery</t>
+          <t>Gossip-Hungry MIL Snoops Through Confidential Files, Learns Attorney DIL Takes Privacy Seriously</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0142-wife-learns-husband-orchestrated-their-relationship-after-sh.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0142-gossip-hungry-mil-snoops-through-confidential-files-learns-a.jpg</t>
         </is>
       </c>
     </row>
@@ -2589,12 +2597,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>MIL Wears White To Wedding, Bride Decides To Make Her The Center Of Attention</t>
+          <t>Sister Assumes She Is Getting Pregnant Teen’s Baby Without Asking, Loses It When The Answer Is No</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0143-mil-wears-white-to-wedding-bride-decides-to-make-her-the-cen.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0143-sister-assumes-she-is-getting-pregnant-teens-baby-without-as.jpg</t>
         </is>
       </c>
     </row>
@@ -2604,12 +2612,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Boyfriend Says Woman Isn’t Worth It Anymore Just Because She Made Her Boundaries Clear</t>
+          <t>Wife Spends Hours Dealing With Drunk Hubby’s Mess, Then Security Footage Changes Everything</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0144-boyfriend-says-woman-isnt-worth-it-anymore-just-because-she-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0144-wife-spends-hours-dealing-with-drunk-hubbys-mess-then-securi.jpg</t>
         </is>
       </c>
     </row>
@@ -2619,12 +2627,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>The Way You Handle Loneliness Says More About You Than You’d Think – Find Out In 27 Questions</t>
+          <t>Woman Tries To Make Sis Feel Bad About Her Past Drinking Problems, Sis Gives Her A Reality Check</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0145-the-way-you-handle-loneliness-says-more-about-you-than-youd-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0145-woman-tries-to-make-sis-feel-bad-about-her-past-drinking-pro.jpg</t>
         </is>
       </c>
     </row>
@@ -2634,12 +2642,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Daily Guess The Country Game #035 (Jun 20, 2026)</t>
+          <t>Daily Guess The Timeline Game #083 (Jun 14, 2026)</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0146-daily-guess-the-country-game-035-jun-20-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0146-daily-guess-the-timeline-game-083-jun-14-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -2649,12 +2657,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Daily Word Search Game #033 (Jun 20, 2026)</t>
+          <t>30 Father’s Day Gifts That Went Completely Off Script And Are Honestly So Much Better For It</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0147-daily-word-search-game-033-jun-20-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0147-30-fathers-day-gifts-that-went-completely-off-script-and-are.jpg</t>
         </is>
       </c>
     </row>
@@ -2664,12 +2672,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Daily Guess The Famous Person Game #094 (Jun 20, 2026)</t>
+          <t>75 Ironic Posts That Might Make You Chuckle</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0148-daily-guess-the-famous-person-game-094-jun-20-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0148-75-ironic-posts-that-might-make-you-chuckle.jpg</t>
         </is>
       </c>
     </row>
@@ -2679,12 +2687,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Experts Solve Botticelli’s Birth Of Venus Side‑Eye Mystery, And The Reason Is Devastating</t>
+          <t>85 Randomly Funny Memes You Probably Haven’t Seen Before</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0149-experts-solve-botticellis-birth-of-venus-sideeye-mystery-and.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0149-85-randomly-funny-memes-you-probably-havent-seen-before.jpg</t>
         </is>
       </c>
     </row>
@@ -2694,12 +2702,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Daily Guess The Timeline Game #088 (Jun 19, 2026)</t>
+          <t>54 Public Monuments That Became Famous For All The Wrong Reasons</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0150-daily-guess-the-timeline-game-088-jun-19-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0150-54-public-monuments-that-became-famous-for-all-the-wrong-rea.jpg</t>
         </is>
       </c>
     </row>
@@ -2709,12 +2717,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>‘Pirates Of The Caribbean’ Made Keira Knightley A Star At 17, Says The Price Was Years Of Therapy</t>
+          <t>81 People Share Photos That Are Almost Too Perfect To Be Real</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0151-pirates-of-the-caribbean-made-keira-knightley-a-star-at-17-s.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0151-81-people-share-photos-that-are-almost-too-perfect-to-be-rea.jpg</t>
         </is>
       </c>
     </row>
@@ -2724,12 +2732,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Why Tech Billionaires No Longer Want Flight Attendants On Their Private Jets</t>
+          <t>“Here To Explain Everything”: 92 Facts And Stories You Might Not Have Heard Of Before</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0152-why-tech-billionaires-no-longer-want-flight-attendants-on-th.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0152-here-to-explain-everything-92-facts-and-stories-you-might-no.jpg</t>
         </is>
       </c>
     </row>
@@ -2739,12 +2747,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Guy Realizes Why Every Vacation Feels More Like Work Than A Holiday</t>
+          <t>41 Misconceptions And Outdated Beliefs People Proudly Corrected</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0153-guy-realizes-why-every-vacation-feels-more-like-work-than-a-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0153-41-misconceptions-and-outdated-beliefs-people-proudly-correc.jpg</t>
         </is>
       </c>
     </row>
@@ -2754,12 +2762,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Wife’s Suggestion Said In Anger Makes Husband Realize He Loves A Tombstone Too Much</t>
+          <t>85 Feminist Posts That Say The Quiet Part Out Loud</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0154-wifes-suggestion-said-in-anger-makes-husband-realize-he-love.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0154-85-feminist-posts-that-say-the-quiet-part-out-loud.jpg</t>
         </is>
       </c>
     </row>
@@ -2769,12 +2777,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>50 Unhinged Screenshots That Accurately Sum Up Online Dating These Days</t>
+          <t>“Why Aren’t Girls Into Me?”: 50 Real Reasons These Incels Are ‘Forever Alone,’ According To Their Friends</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0155-50-unhinged-screenshots-that-accurately-sum-up-online-dating.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0155-why-arent-girls-into-me-50-real-reasons-these-incels-are-for.jpg</t>
         </is>
       </c>
     </row>
@@ -2784,12 +2792,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Biological Parents Of Baby Born To Different Couple Thanks To IVF-Embryo Mix-Up Lose Custody</t>
+          <t>39 Things Americans Barely Notice That Stand Out To Foreign Visitors</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0156-biological-parents-of-baby-born-to-different-couple-thanks-t.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0156-39-things-americans-barely-notice-that-stand-out-to-foreign-.jpg</t>
         </is>
       </c>
     </row>
@@ -2799,12 +2807,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>79 Houses So Weird People Couldn’t Believe They Were Actually For Sale</t>
+          <t>“Sickening”: 47 Times Women Deeply Regretted Looking Through Their Partner’s Phone</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0157-79-houses-so-weird-people-couldnt-believe-they-were-actually.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0157-sickening-47-times-women-deeply-regretted-looking-through-th.jpg</t>
         </is>
       </c>
     </row>
@@ -2814,12 +2822,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Ex-Girlfriend Assumes Her Former Partner Will Help Her Out, Doesn’t Get The Answer She Wanted</t>
+          <t>Woman Is Asked To Help The Sister Who Slept With Her Boyfriend, Family Drama Follows</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0158-ex-girlfriend-assumes-her-former-partner-will-help-her-out-d.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0158-woman-is-asked-to-help-the-sister-who-slept-with-her-boyfrie.jpg</t>
         </is>
       </c>
     </row>
@@ -2829,12 +2837,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>47 People Share The Spiciest And Most Shocking Secrets From Their Jobs</t>
+          <t>“My Girlfriend Broke Her Back. Her Parents’ Response Shocked Me”</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0159-47-people-share-the-spiciest-and-most-shocking-secrets-from-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0159-my-girlfriend-broke-her-back-her-parents-response-shocked-me.jpg</t>
         </is>
       </c>
     </row>
@@ -2844,12 +2852,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>63 Funny And Cute Cat Photos That Might Make You Smile Today (New Pics)</t>
+          <t>Your Social Battery Has A Limit – These 27 Questions Reveal Exactly Where It Is</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0160-63-funny-and-cute-cat-photos-that-might-make-you-smile-today.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0160-your-social-battery-has-a-limit-these-27-questions-reveal-ex.jpg</t>
         </is>
       </c>
     </row>
@@ -2859,12 +2867,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Family Conflict Resolution: 5 Steps to De-escalate Tension at Home</t>
+          <t>Daily Guess The Country Game #029 (Jun 14, 2026)</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0161-family-conflict-resolution-5-steps-to-de-escalate-tension-at.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0161-daily-guess-the-country-game-029-jun-14-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -2874,12 +2882,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>105 Times People Hit The Jackpot While Dumpster Diving (New Pics)</t>
+          <t>Daily Word Search Game #027 (Jun 14, 2026)</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0162-105-times-people-hit-the-jackpot-while-dumpster-diving-new-p.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0162-daily-word-search-game-027-jun-14-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -2889,12 +2897,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Daily Guess The Country Game #034 (Jun 19, 2026)</t>
+          <t>Daily Guess The Famous Person Game #088 (Jun 14, 2026)</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0163-daily-guess-the-country-game-034-jun-19-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0163-daily-guess-the-famous-person-game-088-jun-14-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -2904,12 +2912,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>15 New Comics By Jordan Bolton That Turn Small Encounters Into Heartbreaking Stories</t>
+          <t>Daily Guess The Timeline Game #082 (Jun 13, 2026)</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0164-15-new-comics-by-jordan-bolton-that-turn-small-encounters-in.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0164-daily-guess-the-timeline-game-082-jun-13-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -2919,12 +2927,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Only High IQs Can Beat All 26 Hard General Knowledge Questions – Prove You’re One</t>
+          <t>For Decades, Wives Paid A Mysterious Woman To Fix Their Marriage—Until A Guilt-Ridden Client Told Police All</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0165-only-high-iqs-can-beat-all-26-hard-general-knowledge-questio.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0165-for-decades-wives-paid-a-mysterious-woman-to-fix-their-marri.jpg</t>
         </is>
       </c>
     </row>
@@ -2934,12 +2942,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Through Her Beautiful Driftwood Sculptures, This Artist Seeks To Highlight The Unity Of Human Beings With Nature (28 New Pics)</t>
+          <t>81 Designs So Bad That They Deserve To Be Named And Shamed Online (New Pics)</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0166-through-her-beautiful-driftwood-sculptures-this-artist-seeks.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0166-81-designs-so-bad-that-they-deserve-to-be-named-and-shamed-o.jpg</t>
         </is>
       </c>
     </row>
@@ -2949,12 +2957,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>20 Children’s Drawings Turned Into Handcrafted Enamel Jewelry By Minttnim</t>
+          <t>67 Wholesome Internet Finds That Might Restore Your Faith In Humanity (New Pics)</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0167-20-childrens-drawings-turned-into-handcrafted-enamel-jewelry.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0167-67-wholesome-internet-finds-that-might-restore-your-faith-in.jpg</t>
         </is>
       </c>
     </row>
@@ -2964,12 +2972,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>This Tattoo Artist Was Given A Once-In-A-Lifetime Opportunity At Space Center Houston</t>
+          <t>Someone Asked For Wholesome Pics Of World Leaders, 35 People Share Their Favorites</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0168-this-tattoo-artist-was-given-a-once-in-a-lifetime-opportunit.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0168-someone-asked-for-wholesome-pics-of-world-leaders-35-people-.jpg</t>
         </is>
       </c>
     </row>
@@ -2979,12 +2987,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>‘Best Bird Shots’ 80 Amazing Photos Showing The Beauty Of Wildlife In Detail</t>
+          <t>‘The Weird Unknown’: 79 Creepy, Weird, And Intriguing Facts About The Ocean (New Pics)</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0169-best-bird-shots-80-amazing-photos-showing-the-beauty-of-wild.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0169-the-weird-unknown-79-creepy-weird-and-intriguing-facts-about.jpg</t>
         </is>
       </c>
     </row>
@@ -2994,12 +3002,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>If You Can Name All 25 Characters From These Silhouettes, Your Movie Knowledge Is Next Level</t>
+          <t>People Who Lived Through The 1990s And 2000s Are Thoroughly Enjoying These 121 Posts (New Pics)</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0170-if-you-can-name-all-25-characters-from-these-silhouettes-you.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0170-people-who-lived-through-the-1990s-and-2000s-are-thoroughly-.jpg</t>
         </is>
       </c>
     </row>
@@ -3009,12 +3017,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Daily Word Search Game #032 (Jun 19, 2026)</t>
+          <t>64 Urban Hell Photos That Have People Wondering How These Places Came To Be</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0171-daily-word-search-game-032-jun-19-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0171-64-urban-hell-photos-that-have-people-wondering-how-these-pl.jpg</t>
         </is>
       </c>
     </row>
@@ -3024,12 +3032,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Woman Shares A Pic Of The Dress She Wore To A Wedding And Asks If The Backlash Was Fair</t>
+          <t>45 Times People Asked Dumb Science Questions And The Internet Delivered Perfect Answers</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0172-woman-shares-a-pic-of-the-dress-she-wore-to-a-wedding-and-as.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0172-45-times-people-asked-dumb-science-questions-and-the-interne.jpg</t>
         </is>
       </c>
     </row>
@@ -3039,12 +3047,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>57 Heartwarming Posts From The Better Side Of The Internet</t>
+          <t>65 Men Recall The Exact Moment Everything Fell Apart</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0173-57-heartwarming-posts-from-the-better-side-of-the-internet.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0173-65-men-recall-the-exact-moment-everything-fell-apart.jpg</t>
         </is>
       </c>
     </row>
@@ -3054,12 +3062,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>“Male Karen” Faces Karma After Harassing Dad For Helping Daughters In Women’s Restroom And Making Girl Cry</t>
+          <t>“We Don’t Believe Employees Should Own Pets”: 27 Bosses And Employers That Are Truly The Worst</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0174-male-karen-faces-karma-after-harassing-dad-for-helping-daugh.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0174-we-dont-believe-employees-should-own-pets-27-bosses-and-empl.jpg</t>
         </is>
       </c>
     </row>
@@ -3069,12 +3077,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>“Could You Pass This General Science Quiz?”: Prove Your Brains Can Take It With 20 Questions</t>
+          <t>81 Funny Memes That People In Sales May Use To Explain What They Do To Their Families And Friends</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0175-could-you-pass-this-general-science-quiz-prove-your-brains-c.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0175-81-funny-memes-that-people-in-sales-may-use-to-explain-what-.jpg</t>
         </is>
       </c>
     </row>
@@ -3084,12 +3092,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>55 Terrifying Encounters People Wish They Could Rationally Explain</t>
+          <t>Man Says His Girlfriend Won’t Allow Him To Enter One Room In Her House, Is Shocked To Learn The Truth</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0176-55-terrifying-encounters-people-wish-they-could-rationally-e.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0176-man-says-his-girlfriend-wont-allow-him-to-enter-one-room-in-.jpg</t>
         </is>
       </c>
     </row>
@@ -3099,12 +3107,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Brother’s Fiancée Throws A Full-Blown Tantrum Over A Dress That’s Not Even Hers</t>
+          <t>Bride Starts Having Doubts 9 Days Before The Wedding, Internet Pushes Her To Walk Away Now</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0177-brothers-fiancee-throws-a-full-blown-tantrum-over-a-dress-th.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0177-bride-starts-having-doubts-9-days-before-the-wedding-interne.jpg</t>
         </is>
       </c>
     </row>
@@ -3114,12 +3122,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Daily Guess The Famous Person Game #093 (Jun 19, 2026)</t>
+          <t>Decide If These People Had A Valid Response In 10 Real-Life Situations</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0178-daily-guess-the-famous-person-game-093-jun-19-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0178-decide-if-these-people-had-a-valid-response-in-10-real-life-.jpg</t>
         </is>
       </c>
     </row>
@@ -3129,12 +3137,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>This Artist Turns Family Banter, Bad Luck, And Daily Life Into Colorful Comics (24 New Comics)</t>
+          <t>Daily Guess The Country Game #028 (Jun 13, 2026)</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0179-this-artist-turns-family-banter-bad-luck-and-daily-life-into.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0179-daily-guess-the-country-game-028-jun-13-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -3144,12 +3152,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>“Stands Like A Human”: 35 Surprising Facts And Stories About Animals That Might Teach You Something New</t>
+          <t>Daily Word Search Game #026 (Jun 13, 2026)</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0180-stands-like-a-human-35-surprising-facts-and-stories-about-an.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0180-daily-word-search-game-026-jun-13-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -3159,12 +3167,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>55 Eerie Photos Of Abandoned Places And Forgotten Corners Of America By Brendon Burton</t>
+          <t>Daily Guess The Famous Person Game #087 (Jun 13, 2026)</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0181-55-eerie-photos-of-abandoned-places-and-forgotten-corners-of.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0181-daily-guess-the-famous-person-game-087-jun-13-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -3174,12 +3182,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>“My Wedding Day”: 92 Times People Misread Social Cues So Badly, It Still Hurts To Remember</t>
+          <t>Man Reconnects With A Childhood Friend He Hasn’t Seen In 10 Years, Blows Up The Life He’s Built</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0182-my-wedding-day-92-times-people-misread-social-cues-so-badly-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0182-man-reconnects-with-a-childhood-friend-he-hasnt-seen-in-10-y.jpg</t>
         </is>
       </c>
     </row>
@@ -3189,12 +3197,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>“What’s The Biggest Plot Twist In History?” (32 Posts)</t>
+          <t>Bride Bans Sister’s Boyfriend From Wedding For Disgusting And Ridiculous Reasons</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0183-whats-the-biggest-plot-twist-in-history-32-posts.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0183-bride-bans-sisters-boyfriend-from-wedding-for-disgusting-and.jpg</t>
         </is>
       </c>
     </row>
@@ -3204,12 +3212,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>66 Poorly Designed Signs That Resulted In Hilarious Messages (New Pics)</t>
+          <t>Ben Stiller Faces Backlash After Viral Video Appears To Contradict His Message On Homelessness</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0184-66-poorly-designed-signs-that-resulted-in-hilarious-messages.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0184-ben-stiller-faces-backlash-after-viral-video-appears-to-cont.jpg</t>
         </is>
       </c>
     </row>
@@ -3219,12 +3227,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Toxic Neighbor Learns $437K Lesson After Destroying Historic Orchard, Loses Her Home In The Process</t>
+          <t>40 Funny Pics Of Cats Being Themselves And Showing Off Their Shredded Masterpieces</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0185-toxic-neighbor-learns-437k-lesson-after-destroying-historic-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0185-40-funny-pics-of-cats-being-themselves-and-showing-off-their.jpg</t>
         </is>
       </c>
     </row>
@@ -3234,12 +3242,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Teen Survives Being Kicked Out By Her Dad, Her Comeback Is So Remarkable He Is Now The One Begging</t>
+          <t>34 Scam Examples That Show America Is Living In A Completely Different Reality From Everyone Else</t>
         </is>
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0186-teen-survives-being-kicked-out-by-her-dad-her-comeback-is-so.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0186-34-scam-examples-that-show-america-is-living-in-a-completely.jpg</t>
         </is>
       </c>
     </row>
@@ -3249,12 +3257,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Company Pins Missing $361 On The New Guy, Watches Thousands Go Up In Smoke When He Starts Talking</t>
+          <t>“Thank You Wave In Traffic”: 59 Social Contracts That Make Everyday Life Better</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0187-company-pins-missing-361-on-the-new-guy-watches-thousands-go.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0187-thank-you-wave-in-traffic-59-social-contracts-that-make-ever.jpg</t>
         </is>
       </c>
     </row>
@@ -3264,12 +3272,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Teacher Refuses To Change Attendance Policy Even For 11YO’s Chemotherapy, Mom Takes Her Anger Online</t>
+          <t>Looksmaxxer Clavicular Just Had His 3rd Surgery, And People Are Getting Concerned About His Transformation</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0188-teacher-refuses-to-change-attendance-policy-even-for-11yos-c.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0188-looksmaxxer-clavicular-just-had-his-3rd-surgery-and-people-a.jpg</t>
         </is>
       </c>
     </row>
@@ -3279,12 +3287,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Woman Says Husband’s Car Triggers Panic Attacks, Asks Couple To Text Before Leaving Home</t>
+          <t>“Do You Understand How The Body Works?”: Score 20/24 To Prove It In This Biology Quiz</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0189-woman-says-husbands-car-triggers-panic-attacks-asks-couple-t.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0189-do-you-understand-how-the-body-works-score-2024-to-prove-it-.jpg</t>
         </is>
       </c>
     </row>
@@ -3294,12 +3302,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Surf Instructor Claps Back After Karen Demands She Cover Up Because Her Tween Feels Self-Conscious</t>
+          <t>59 Design Disasters That Are So Bad, They’re Honestly Kind Of Funny (New Pics)</t>
         </is>
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0190-surf-instructor-claps-back-after-karen-demands-she-cover-up-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0190-59-design-disasters-that-are-so-bad-theyre-honestly-kind-of-.jpg</t>
         </is>
       </c>
     </row>
@@ -3309,12 +3317,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Guy Lies About Allergy While On Tinder Date, Ends Up At The Emergency Room With $500 Bill</t>
+          <t>83 Examples Of “Awful Taste But Great Execution” That Left People Confused (New Pics)</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0191-guy-lies-about-allergy-while-on-tinder-date-ends-up-at-the-e.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0191-83-examples-of-awful-taste-but-great-execution-that-left-peo.jpg</t>
         </is>
       </c>
     </row>
@@ -3324,12 +3332,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Guy Loses Trust In Wife After Living With The Consequences Of Her Impulsive Decisions For 10 Years</t>
+          <t>46 Times People Heard Such Genius Insults They Memorized Them</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0192-guy-loses-trust-in-wife-after-living-with-the-consequences-o.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0192-46-times-people-heard-such-genius-insults-they-memorized-the.jpg</t>
         </is>
       </c>
     </row>
@@ -3339,12 +3347,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>“Lost A Bet With The Fashion Gods”: 20 Celebrity Outfits Compared With Their Original Runway Versions</t>
+          <t>63 Photos That Are So Great, They Deserve To Be Seen By More People</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0193-lost-a-bet-with-the-fashion-gods-20-celebrity-outfits-compar.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0193-63-photos-that-are-so-great-they-deserve-to-be-seen-by-more-.jpg</t>
         </is>
       </c>
     </row>
@@ -3354,12 +3362,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>A Guy Stole His Best Friend’s 8-Month Project Car Profit For A Bali Trip, Until A Text Trapped Him</t>
+          <t>Bride’s Wedding Guests Start Canceling One By One, The Reason Why Leaves Her Speechless</t>
         </is>
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0194-a-guy-stole-his-best-friends-8-month-project-car-profit-for-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0194-brides-wedding-guests-start-canceling-one-by-one-the-reason-.jpg</t>
         </is>
       </c>
     </row>
@@ -3369,12 +3377,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>“They Don’t Eat Leftovers”: 56 Ignorant Middle-Class Phrases That They Need To Rethink</t>
+          <t>Woman Calls The Police After Learning What Her Sister Served For Lunch</t>
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0195-they-dont-eat-leftovers-56-ignorant-middle-class-phrases-tha.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0195-woman-calls-the-police-after-learning-what-her-sister-served.jpg</t>
         </is>
       </c>
     </row>
@@ -3384,12 +3392,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>“Are You A Geography Genius?”: Identify The Location Of These 19 Famous Places To Prove It</t>
+          <t>Toxic Fiancée Airs All Their Dirty Laundry, Guy’s Friends Finally Decide To Break Their Silence</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0196-are-you-a-geography-genius-identify-the-location-of-these-19.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0196-toxic-fiancee-airs-all-their-dirty-laundry-guys-friends-fina.jpg</t>
         </is>
       </c>
     </row>
@@ -3399,12 +3407,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>67 Couches That Raise More Questions Than Any Piece Of Furniture Ever Should</t>
+          <t>From Hidden Objects To Impossible Perspectives: Challenge Your Vision With 15 Image Riddles</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0197-67-couches-that-raise-more-questions-than-any-piece-of-furni.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0197-from-hidden-objects-to-impossible-perspectives-challenge-you.jpg</t>
         </is>
       </c>
     </row>
@@ -3414,12 +3422,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Margot Robbie Lost Her Cool When She Found Out Her Husband Was In Harry Potter Before They Met</t>
+          <t>Doctor Warns Of The Risks After “Looksmaxxer” Films Himself Using A Maxilla Expander</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0198-margot-robbie-lost-her-cool-when-she-found-out-her-husband-w.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0198-doctor-warns-of-the-risks-after-looksmaxxer-films-himself-us.jpg</t>
         </is>
       </c>
     </row>
@@ -3429,12 +3437,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>76 People Who Had The Audacity To Do What Everyone Else Was Thinking</t>
+          <t>29 Amazing Wall Transformations By Nuno Miles That Turn Urban Spaces Into Hyperrealistic Art</t>
         </is>
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0199-76-people-who-had-the-audacity-to-do-what-everyone-else-was-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0199-29-amazing-wall-transformations-by-nuno-miles-that-turn-urba.jpg</t>
         </is>
       </c>
     </row>
@@ -3444,12 +3452,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>“I’m Personally 99% Against”: Uncle’s ‘Paranoid’ Advice To Niece Turns Out To Be A Life Saver</t>
+          <t>Daily Word Search Game #025 (Jun 12, 2026)</t>
         </is>
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/T/pins/0200-im-personally-99-against-uncles-paranoid-advice-to-niece-tur.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0200-daily-word-search-game-025-jun-12-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -3546,114 +3554,115 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId200"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add pins - 2026-07-16 08:03 UTC
</commit_message>
<xml_diff>
--- a/pins/pin_links.xlsx
+++ b/pins/pin_links.xlsx
@@ -752,12 +752,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Groom Promises All 3 Sisters Bridesmaid Dresses, Bride Hands Out Rejection Letters Based On Weight</t>
+          <t>Sister Learns She’s No Longer In Brother’s Wedding Party, Heartbroken By Bride’s Explanation</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0020-groom-promises-all-3-sisters-bridesmaid-dresses-bride-hands-.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0020-sister-learns-shes-no-longer-in-brothers-wedding-party-heart.jpg</t>
         </is>
       </c>
     </row>
@@ -767,12 +767,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Entitled Influencers Try To Use Luxe Hotel For Insta Pics, Badmouth The Venue When They’re Sent Home</t>
+          <t>Influencers Want Five-Star Content On A Zero-Star Budget, Luxury Hotel Finally Stops Playing Along</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0021-entitled-influencers-try-to-use-luxe-hotel-for-insta-pics-ba.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0021-influencers-want-five-star-content-on-a-zero-star-budget-lux.jpg</t>
         </is>
       </c>
     </row>
@@ -782,12 +782,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Student Blames Everyone Around But Himself In His Failures, Demands A Solo Project And Fails Again</t>
+          <t>Stubborn Student Refuses To Work In A Group Despite Professor’s Warnings, Regrets It When He Fails</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0022-student-blames-everyone-around-but-himself-in-his-failures-d.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0022-stubborn-student-refuses-to-work-in-a-group-despite-professo.jpg</t>
         </is>
       </c>
     </row>
@@ -797,12 +797,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>77 Quick, Clever, And Unexpected Comics From Joe Lennon (New Pics)</t>
+          <t>Life Is Weird And Hilarious: 77 New One-Panel Comics From Joe Lennon</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0023-77-quick-clever-and-unexpected-comics-from-joe-lennon-new-pi.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0023-life-is-weird-and-hilarious-77-new-one-panel-comics-from-joe.jpg</t>
         </is>
       </c>
     </row>
@@ -812,12 +812,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Boyfriend Secretly Blocks Woman’s Male Friends On Facebook, Claims It’s Just Being “Protective”</t>
+          <t>BF Thinks He’s Entitled To Block GF’s Male Friends On Her Behalf, Fumes As She Leaves Him Over It</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0024-boyfriend-secretly-blocks-womans-male-friends-on-facebook-cl.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0024-bf-thinks-hes-entitled-to-block-gfs-male-friends-on-her-beha.jpg</t>
         </is>
       </c>
     </row>
@@ -827,12 +827,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Struggling Dad Blames Wife For Sixth Pregnancy, Brother Gives Him A Brutal Reality Check</t>
+          <t>Bro Refuses To Sit Quietly While His Sibling Blames His Wife For Their Sixth Child And Money Woes</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0025-struggling-dad-blames-wife-for-sixth-pregnancy-brother-gives.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0025-bro-refuses-to-sit-quietly-while-his-sibling-blames-his-wife.jpg</t>
         </is>
       </c>
     </row>
@@ -842,12 +842,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IT Worker Takes Down Buffoon Accountant With Clever Plan, Says “Network’s Down” Right Back At Her</t>
+          <t>Accounting Manager Turns IT Guy’s Work Life Into A Nightmare, His Epic Revenge Leaves Her Jobless</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0026-it-worker-takes-down-buffoon-accountant-with-clever-plan-say.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0026-accounting-manager-turns-it-guys-work-life-into-a-nightmare-.jpg</t>
         </is>
       </c>
     </row>
@@ -872,12 +872,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>From Sand To Packaging, Here Are 34 Unpopular Industries That Actually Make Millions</t>
+          <t>34 Secretive And Weird Billion-Dollar Industries Revealed Online That Most People Never Hear About</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0028-from-sand-to-packaging-here-are-34-unpopular-industries-that.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0028-34-secretive-and-weird-billion-dollar-industries-revealed-on.jpg</t>
         </is>
       </c>
     </row>
@@ -887,12 +887,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Woman Serves Mean Teammates The Best Brownies Ever, Keeps Her Recipe Secret As Petty Payback</t>
+          <t>Woman Serves Horrible Teammates Amazing Brownies, Keeps The Secret Locked Up As The Best Payback</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0029-woman-serves-mean-teammates-the-best-brownies-ever-keeps-her.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0029-woman-serves-horrible-teammates-amazing-brownies-keeps-the-s.jpg</t>
         </is>
       </c>
     </row>
@@ -1007,12 +1007,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Wordle #1851: Hints &amp; Answer (Jul 14, 2026)</t>
+          <t>Wordle #1852: Hints &amp; Answer (Jul 15, 2026)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0037-wordle-1851-hints-answer-jul-14-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0037-wordle-1852-hints-answer-jul-15-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -2130,16 +2130,8 @@
       <c r="A113" t="n">
         <v>112</v>
       </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>Striking Comparison Between Charlize Theron And Anne Hathaway Provokes Discussion On Beauty Standards</t>
-        </is>
-      </c>
-      <c r="C113" s="2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0112-striking-comparison-between-charlize-theron-and-anne-hathawa.jpg</t>
-        </is>
-      </c>
+      <c r="B113" t="inlineStr"/>
+      <c r="C113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -8074,395 +8066,394 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId109"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C207" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C208" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C209" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C210" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C220" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C221" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C222" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C223" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C224" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C225" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C226" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C227" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C228" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C229" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C230" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C231" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C232" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C233" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C234" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C235" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C236" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C237" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C238" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C239" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C240" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C241" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C242" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C243" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C244" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C245" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C246" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C247" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C248" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C249" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C250" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C251" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C252" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C253" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C254" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C255" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C256" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C257" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C258" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C259" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C260" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C261" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C262" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C263" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C264" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C265" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C266" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C267" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C268" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C269" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C270" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C271" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C272" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C273" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C274" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C275" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C276" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C277" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C278" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C279" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C280" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C281" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C282" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C283" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C284" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C285" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C286" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C287" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C288" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C289" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C290" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C291" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C292" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C293" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C294" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C295" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C296" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C297" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C298" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C299" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C300" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C301" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C302" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C303" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C304" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C305" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C306" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C307" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C308" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C309" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C310" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C311" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C312" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C313" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C314" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C315" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C316" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C317" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C318" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C319" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C320" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C321" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C322" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C323" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C324" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C325" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C326" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C327" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C328" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C329" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C330" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C331" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C332" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C333" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C334" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C335" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C336" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C337" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C338" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C339" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C340" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C341" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C342" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C343" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C344" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C345" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C346" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C347" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C348" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C349" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C350" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C351" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C352" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C353" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C354" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C355" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C356" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C357" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C358" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C359" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C360" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C361" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C362" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C363" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C364" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C365" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C366" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C367" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C368" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C369" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C370" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C371" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C372" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C373" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C374" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C375" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C376" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C377" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C378" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C379" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C380" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C381" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C382" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C383" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C384" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C385" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C386" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C387" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C388" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C389" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C390" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C391" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C392" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C393" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C394" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C395" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C396" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C397" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C398" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C399" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C400" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C401" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C402" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C403" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C404" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C405" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C406" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C407" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C408" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C409" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C410" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C411" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C412" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C413" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C414" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C415" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C416" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C417" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C418" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C419" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C420" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C421" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C422" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C423" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C424" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C425" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C426" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C427" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C428" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C429" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C430" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C431" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C432" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C433" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C434" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C435" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C436" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C437" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C438" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C439" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C440" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C441" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C442" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C443" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C444" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C445" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C446" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C447" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C448" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C449" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C450" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C451" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C452" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C453" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C454" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C455" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C456" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C457" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C458" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C459" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C460" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C461" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C462" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C463" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C464" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C465" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C466" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C467" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C468" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C469" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C470" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C471" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C472" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C473" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C474" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C475" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C476" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C477" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C478" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C479" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C480" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C481" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C482" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C483" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C484" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C485" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C486" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C487" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C488" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C489" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C490" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C491" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C492" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C493" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C494" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C495" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C496" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C497" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C498" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C499" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C500" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C501" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C207" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C208" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C209" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C210" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C220" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C221" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C222" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C223" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C224" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C225" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C226" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C227" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C228" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C229" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C230" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C231" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C232" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C233" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C234" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C235" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C236" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C237" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C238" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C239" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C240" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C241" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C242" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C243" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C244" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C245" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C246" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C247" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C248" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C249" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C250" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C251" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C252" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C253" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C254" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C255" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C256" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C257" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C258" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C259" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C260" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C261" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C262" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C263" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C264" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C265" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C266" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C267" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C268" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C269" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C270" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C271" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C272" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C273" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C274" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C275" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C276" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C277" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C278" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C279" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C280" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C281" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C282" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C283" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C284" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C285" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C286" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C287" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C288" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C289" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C290" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C291" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C292" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C293" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C294" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C295" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C296" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C297" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C298" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C299" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C300" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C301" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C302" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C303" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C304" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C305" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C306" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C307" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C308" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C309" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C310" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C311" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C312" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C313" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C314" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C315" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C316" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C317" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C318" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C319" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C320" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C321" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C322" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C323" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C324" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C325" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C326" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C327" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C328" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C329" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C330" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C331" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C332" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C333" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C334" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C335" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C336" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C337" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C338" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C339" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C340" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C341" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C342" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C343" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C344" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C345" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C346" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C347" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C348" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C349" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C350" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C351" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C352" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C353" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C354" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C355" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C356" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C357" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C358" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C359" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C360" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C361" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C362" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C363" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C364" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C365" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C366" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C367" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C368" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C369" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C370" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C371" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C372" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C373" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C374" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C375" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C376" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C377" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C378" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C379" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C380" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C381" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C382" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C383" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C384" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C385" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C386" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C387" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C388" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C389" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C390" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C391" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C392" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C393" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C394" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C395" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C396" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C397" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C398" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C399" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C400" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C401" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C402" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C403" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C404" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C405" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C406" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C407" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C408" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C409" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C410" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C411" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C412" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C413" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C414" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C415" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C416" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C417" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C418" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C419" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C420" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C421" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C422" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C423" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C424" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C425" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C426" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C427" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C428" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C429" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C430" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C431" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C432" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C433" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C434" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C435" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C436" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C437" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C438" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C439" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C440" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C441" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C442" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C443" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C444" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C445" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C446" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C447" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C448" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C449" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C450" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C451" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C452" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C453" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C454" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C455" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C456" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C457" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C458" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C459" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C460" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C461" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C462" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C463" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C464" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C465" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C466" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C467" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C468" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C469" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C470" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C471" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C472" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C473" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C474" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C475" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C476" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C477" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C478" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C479" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C480" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C481" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C482" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C483" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C484" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C485" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C486" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C487" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C488" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C489" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C490" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C491" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C492" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C493" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C494" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C495" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C496" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C497" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C498" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C499" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C500" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C501" r:id="rId499"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add pins - 2026-07-17 07:59 UTC
</commit_message>
<xml_diff>
--- a/pins/pin_links.xlsx
+++ b/pins/pin_links.xlsx
@@ -2130,8 +2130,16 @@
       <c r="A113" t="n">
         <v>112</v>
       </c>
-      <c r="B113" t="inlineStr"/>
-      <c r="C113" t="inlineStr"/>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Striking Comparison Between Charlize Theron And Anne Hathaway Provokes Discussion On Beauty Standards</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0112-striking-comparison-between-charlize-theron-and-anne-hathawa.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -3847,16 +3855,8 @@
       <c r="A228" t="n">
         <v>227</v>
       </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>Biohacker Bryan Johnson Reveals Dreadful Diagnosis Despite Meticulous And Intense Health Regimen</t>
-        </is>
-      </c>
-      <c r="C228" s="2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0227-biohacker-bryan-johnson-reveals-dreadful-diagnosis-despite-m.jpg</t>
-        </is>
-      </c>
+      <c r="B228" t="inlineStr"/>
+      <c r="C228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -8066,121 +8066,121 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId109"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C207" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C208" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C209" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C210" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C220" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C221" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C222" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C223" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C224" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C225" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C226" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C227" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C228" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C207" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C208" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C209" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C210" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C220" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C221" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C222" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C223" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C224" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C225" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C226" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C227" r:id="rId226"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C229" r:id="rId227"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C230" r:id="rId228"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C231" r:id="rId229"/>

</xml_diff>

<commit_message>
Add pins - 2026-07-18 07:39 UTC
</commit_message>
<xml_diff>
--- a/pins/pin_links.xlsx
+++ b/pins/pin_links.xlsx
@@ -690,16 +690,8 @@
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>24 Award-Winning Wildlife Photos Shared By The Artist Gallery</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0016-24-award-winning-wildlife-photos-shared-by-the-artist-galler.jpg</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1007,12 +999,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Wordle #1852: Hints &amp; Answer (Jul 15, 2026)</t>
+          <t>Wordle #1854: Hints &amp; Answer (Jul 17, 2026)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0037-wordle-1852-hints-answer-jul-15-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0037-wordle-1854-hints-answer-jul-17-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -3855,8 +3847,16 @@
       <c r="A228" t="n">
         <v>227</v>
       </c>
-      <c r="B228" t="inlineStr"/>
-      <c r="C228" t="inlineStr"/>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Biohacker Bryan Johnson Reveals Dreadful Diagnosis Despite Meticulous And Intense Health Regimen</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0227-biohacker-bryan-johnson-reveals-dreadful-diagnosis-despite-m.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -7970,217 +7970,217 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C207" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C208" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C209" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C210" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C220" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C221" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C222" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C223" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C224" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C225" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C226" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C227" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C207" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C208" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C209" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C210" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C220" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C221" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C222" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C223" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C224" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C225" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C226" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C227" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C228" r:id="rId226"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C229" r:id="rId227"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C230" r:id="rId228"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C231" r:id="rId229"/>

</xml_diff>

<commit_message>
Add pins - 2026-07-19 08:10 UTC
</commit_message>
<xml_diff>
--- a/pins/pin_links.xlsx
+++ b/pins/pin_links.xlsx
@@ -690,8 +690,16 @@
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>24 Award-Winning Wildlife Photos Shared By The Artist Gallery</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0016-24-award-winning-wildlife-photos-shared-by-the-artist-galler.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -999,12 +1007,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Wordle #1854: Hints &amp; Answer (Jul 17, 2026)</t>
+          <t>Wordle #1855: Hints &amp; Answer (Jul 18, 2026)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0037-wordle-1854-hints-answer-jul-17-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0037-wordle-1855-hints-answer-jul-18-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -7970,490 +7978,491 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C207" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C208" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C209" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C210" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C220" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C221" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C222" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C223" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C224" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C225" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C226" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C227" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C228" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C229" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C230" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C231" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C232" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C233" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C234" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C235" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C236" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C237" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C238" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C239" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C240" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C241" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C242" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C243" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C244" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C245" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C246" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C247" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C248" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C249" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C250" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C251" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C252" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C253" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C254" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C255" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C256" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C257" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C258" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C259" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C260" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C261" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C262" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C263" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C264" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C265" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C266" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C267" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C268" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C269" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C270" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C271" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C272" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C273" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C274" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C275" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C276" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C277" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C278" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C279" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C280" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C281" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C282" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C283" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C284" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C285" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C286" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C287" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C288" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C289" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C290" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C291" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C292" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C293" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C294" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C295" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C296" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C297" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C298" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C299" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C300" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C301" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C302" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C303" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C304" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C305" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C306" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C307" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C308" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C309" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C310" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C311" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C312" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C313" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C314" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C315" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C316" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C317" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C318" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C319" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C320" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C321" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C322" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C323" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C324" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C325" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C326" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C327" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C328" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C329" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C330" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C331" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C332" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C333" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C334" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C335" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C336" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C337" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C338" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C339" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C340" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C341" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C342" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C343" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C344" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C345" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C346" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C347" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C348" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C349" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C350" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C351" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C352" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C353" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C354" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C355" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C356" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C357" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C358" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C359" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C360" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C361" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C362" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C363" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C364" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C365" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C366" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C367" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C368" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C369" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C370" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C371" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C372" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C373" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C374" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C375" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C376" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C377" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C378" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C379" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C380" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C381" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C382" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C383" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C384" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C385" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C386" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C387" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C388" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C389" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C390" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C391" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C392" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C393" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C394" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C395" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C396" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C397" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C398" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C399" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C400" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C401" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C402" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C403" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C404" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C405" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C406" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C407" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C408" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C409" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C410" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C411" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C412" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C413" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C414" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C415" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C416" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C417" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C418" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C419" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C420" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C421" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C422" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C423" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C424" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C425" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C426" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C427" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C428" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C429" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C430" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C431" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C432" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C433" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C434" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C435" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C436" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C437" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C438" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C439" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C440" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C441" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C442" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C443" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C444" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C445" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C446" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C447" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C448" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C449" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C450" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C451" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C452" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C453" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C454" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C455" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C456" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C457" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C458" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C459" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C460" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C461" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C462" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C463" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C464" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C465" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C466" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C467" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C468" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C469" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C470" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C471" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C472" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C473" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C474" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C475" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C476" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C477" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C478" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C479" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C480" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C481" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C482" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C483" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C484" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C485" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C486" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C487" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C488" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C489" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C490" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C491" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C492" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C493" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C494" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C495" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C496" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C497" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C498" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C499" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C500" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C501" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C207" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C208" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C209" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C210" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C220" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C221" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C222" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C223" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C224" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C225" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C226" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C227" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C228" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C229" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C230" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C231" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C232" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C233" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C234" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C235" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C236" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C237" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C238" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C239" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C240" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C241" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C242" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C243" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C244" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C245" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C246" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C247" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C248" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C249" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C257" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C258" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C259" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C260" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C267" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C268" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C269" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C270" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C271" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C272" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C273" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C274" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C275" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C276" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C277" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C278" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C279" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C280" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C281" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C282" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C283" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C284" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C285" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C286" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C287" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C288" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C289" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C290" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C291" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C292" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C293" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C294" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C295" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C296" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C297" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C298" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C299" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C300" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C301" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C302" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C303" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C304" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C305" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C306" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C307" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C308" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C309" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C310" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C311" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C312" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C313" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C314" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C315" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C316" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C317" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C318" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C319" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C320" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C321" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C322" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C323" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C324" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C325" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C326" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C327" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C328" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C329" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C330" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C331" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C332" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C333" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C334" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C335" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C336" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C337" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C338" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C339" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C340" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C341" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C342" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C343" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C344" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C345" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C346" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C347" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C348" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C349" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C350" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C351" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C352" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C353" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C354" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C355" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C356" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C357" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C358" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C359" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C360" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C361" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C362" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C363" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C364" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C365" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C366" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C367" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C368" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C369" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C370" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C371" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C372" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C373" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C374" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C375" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C376" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C377" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C378" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C379" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C380" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C381" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C382" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C383" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C384" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C385" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C386" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C387" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C388" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C389" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C390" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C391" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C392" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C393" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C394" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C395" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C396" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C397" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C398" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C399" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C400" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C401" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C402" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C403" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C404" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C405" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C406" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C407" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C408" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C409" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C410" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C411" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C412" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C413" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C414" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C415" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C416" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C417" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C418" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C419" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C420" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C421" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C422" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C423" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C424" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C425" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C426" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C427" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C428" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C429" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C430" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C431" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C432" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C433" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C434" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C435" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C436" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C437" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C438" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C439" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C440" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C441" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C442" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C443" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C444" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C445" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C446" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C447" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C448" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C449" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C450" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C451" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C452" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C453" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C454" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C455" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C456" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C457" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C458" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C459" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C460" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C461" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C462" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C463" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C464" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C465" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C466" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C467" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C468" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C469" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C470" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C471" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C472" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C473" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C474" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C475" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C476" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C477" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C478" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C479" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C480" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C481" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C482" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C483" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C484" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C485" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C486" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C487" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C488" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C489" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C490" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C491" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C492" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C493" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C494" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C495" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C496" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C497" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C498" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C499" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C500" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C501" r:id="rId500"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add pins - 2026-07-20 08:50 UTC
</commit_message>
<xml_diff>
--- a/pins/pin_links.xlsx
+++ b/pins/pin_links.xlsx
@@ -570,16 +570,8 @@
       <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Adult Star Bonnie Blue Describes How Participants Dealt With Her Baby Bump During 10-Hour July 4 Event</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0008-adult-star-bonnie-blue-describes-how-participants-dealt-with.jpg</t>
-        </is>
-      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1007,12 +999,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Wordle #1855: Hints &amp; Answer (Jul 18, 2026)</t>
+          <t>Wordle #1857: Hints &amp; Answer (Jul 20, 2026)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0037-wordle-1855-hints-answer-jul-18-2026.jpg</t>
+          <t>https://raw.githubusercontent.com/Arslan0070/Pins/main/pins/0037-wordle-1857-hints-answer-jul-20-2026.jpg</t>
         </is>
       </c>
     </row>
@@ -7970,499 +7962,498 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C207" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C208" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C209" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C210" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C220" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C221" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C222" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C223" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C224" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C225" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C226" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C227" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C228" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C229" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C230" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C231" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C232" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C233" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C234" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C235" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C236" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C237" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C238" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C239" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C240" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C241" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C242" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C243" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C244" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C245" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C246" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C247" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C248" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C249" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C250" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C251" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C252" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C253" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C254" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C255" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C256" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C257" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C258" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C259" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C260" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C261" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C262" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C263" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C264" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C265" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C266" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C267" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C268" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C269" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C270" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C271" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C272" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C273" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C274" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C275" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C276" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C277" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C278" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C279" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C280" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C281" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C282" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C283" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C284" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C285" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C286" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C287" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C288" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C289" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C290" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C291" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C292" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C293" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C294" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C295" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C296" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C297" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C298" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C299" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C300" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C301" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C302" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C303" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C304" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C305" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C306" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C307" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C308" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C309" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C310" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C311" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C312" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C313" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C314" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C315" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C316" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C317" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C318" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C319" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C320" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C321" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C322" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C323" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C324" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C325" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C326" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C327" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C328" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C329" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C330" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C331" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C332" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C333" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C334" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C335" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C336" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C337" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C338" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C339" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C340" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C341" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C342" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C343" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C344" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C345" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C346" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C347" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C348" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C349" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C350" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C351" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C352" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C353" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C354" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C355" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C356" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C357" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C358" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C359" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C360" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C361" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C362" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C363" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C364" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C365" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C366" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C367" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C368" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C369" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C370" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C371" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C372" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C373" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C374" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C375" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C376" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C377" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C378" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C379" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C380" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C381" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C382" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C383" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C384" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C385" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C386" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C387" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C388" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C389" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C390" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C391" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C392" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C393" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C394" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C395" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C396" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C397" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C398" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C399" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C400" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C401" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C402" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C403" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C404" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C405" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C406" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C407" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C408" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C409" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C410" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C411" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C412" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C413" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C414" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C415" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C416" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C417" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C418" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C419" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C420" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C421" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C422" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C423" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C424" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C425" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C426" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C427" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C428" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C429" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C430" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C431" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C432" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C433" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C434" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C435" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C436" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C437" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C438" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C439" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C440" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C441" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C442" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C443" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C444" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C445" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C446" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C447" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C448" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C449" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C450" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C451" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C452" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C453" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C454" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C455" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C456" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C457" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C458" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C459" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C460" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C461" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C462" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C463" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C464" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C465" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C466" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C467" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C468" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C469" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C470" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C471" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C472" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C473" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C474" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C475" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C476" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C477" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C478" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C479" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C480" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C481" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C482" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C483" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C484" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C485" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C486" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C487" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C488" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C489" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C490" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C491" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C492" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C493" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C494" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C495" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C496" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C497" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C498" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C499" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C500" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C501" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C207" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C208" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C209" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C210" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C220" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C221" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C222" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C223" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C224" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C225" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C226" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C227" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C228" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C229" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C230" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C231" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C232" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C233" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C234" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C235" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C236" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C237" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C238" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C239" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C240" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C241" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C242" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C243" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C244" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C245" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C246" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C247" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C248" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C249" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C250" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C251" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C252" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C253" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C254" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C255" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C256" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C257" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C258" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C259" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C260" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C261" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C262" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C263" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C264" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C265" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C266" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C267" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C268" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C269" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C270" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C271" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C272" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C273" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C274" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C275" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C276" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C277" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C278" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C279" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C280" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C281" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C282" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C283" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C284" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C285" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C286" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C287" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C288" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C289" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C290" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C291" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C292" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C293" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C294" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C295" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C296" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C297" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C298" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C299" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C300" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C301" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C302" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C303" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C304" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C305" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C306" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C307" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C308" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C309" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C310" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C311" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C312" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C313" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C314" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C315" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C316" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C317" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C318" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C319" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C320" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C321" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C322" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C323" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C324" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C325" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C326" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C327" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C328" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C329" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C330" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C331" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C332" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C333" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C334" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C335" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C336" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C337" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C338" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C339" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C340" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C341" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C342" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C343" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C344" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C345" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C346" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C347" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C348" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C349" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C350" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C351" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C352" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C353" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C354" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C355" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C356" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C357" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C358" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C359" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C360" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C361" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C362" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C363" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C364" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C365" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C366" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C367" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C368" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C369" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C370" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C371" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C372" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C373" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C374" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C375" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C376" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C377" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C378" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C379" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C380" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C381" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C382" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C383" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C384" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C385" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C386" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C387" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C388" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C389" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C390" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C391" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C392" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C393" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C394" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C395" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C396" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C397" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C398" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C399" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C400" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C401" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C402" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C403" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C404" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C405" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C406" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C407" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C408" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C409" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C410" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C411" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C412" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C413" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C414" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C415" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C416" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C417" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C418" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C419" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C420" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C421" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C422" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C423" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C424" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C425" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C426" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C427" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C428" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C429" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C430" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C431" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C432" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C433" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C434" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C435" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C436" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C437" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C438" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C439" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C440" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C441" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C442" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C443" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C444" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C445" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C446" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C447" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C448" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C449" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C450" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C451" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C452" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C453" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C454" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C455" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C456" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C457" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C458" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C459" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C460" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C461" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C462" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C463" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C464" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C465" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C466" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C467" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C468" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C469" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C470" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C471" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C472" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C473" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C474" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C475" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C476" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C477" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C478" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C479" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C480" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C481" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C482" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C483" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C484" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C485" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C486" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C487" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C488" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C489" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C490" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C491" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C492" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C493" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C494" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C495" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C496" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C497" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C498" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C499" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C500" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C501" r:id="rId499"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>